<commit_message>
fix: prevent skipping feedback and stabilize post-submission transitions
</commit_message>
<xml_diff>
--- a/開発進捗管理.xlsx
+++ b/開発進捗管理.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="進捗サマリー" sheetId="1" r:id="R8c2b181042484d8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="実装タスク" sheetId="2" r:id="R7fb24257b8134f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新履歴" sheetId="5" r:id="R288bb67059c445b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="進捗サマリー" sheetId="1" r:id="Rc3ec61def1704ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="実装タスク" sheetId="2" r:id="Rdc585897afa5429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新履歴" sheetId="5" r:id="Rd1ff3e0bdd9c4670"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="207" formatCode="m/d"/>
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="32">
+  <x:fonts count="35">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -202,6 +202,24 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF23423B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF536B63"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF536B63"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -463,7 +481,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="233">
+  <x:cellXfs count="237">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1002,6 +1020,18 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1138,7 +1168,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ProgressHistory" displayName="ProgressHistory" ref="A3:F19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ProgressHistory" displayName="ProgressHistory" ref="A3:F21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="更新日"/>
     <x:tableColumn id="2" name="カテゴリ"/>
@@ -1432,12 +1462,12 @@
       <x:c r="D5" s="200" t="str"/>
       <x:c r="E5" s="201" t="n">
         <x:f>COUNTIF('実装タスク'!$F$5:$F$96,"進行中")</x:f>
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F5" s="200" t="str"/>
       <x:c r="G5" s="201" t="n">
         <x:f>COUNTIF('実装タスク'!$F$5:$F$96,"要確認")</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H5" s="200" t="str"/>
       <x:c r="I5" s="190" t="n">
@@ -1538,7 +1568,7 @@
       </x:c>
       <x:c r="C10" s="38" t="n">
         <x:f>COUNTIFS('実装タスク'!$C$5:$C$96,$A10,'実装タスク'!$F$5:$F$96,"進行中")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="38" t="n">
         <x:f>COUNTIFS('実装タスク'!$C$5:$C$96,$A10,'実装タスク'!$F$5:$F$96,"未着手")</x:f>
@@ -1546,7 +1576,7 @@
       </x:c>
       <x:c r="E10" s="38" t="n">
         <x:f>COUNTIFS('実装タスク'!$C$5:$C$96,$A10,'実装タスク'!$F$5:$F$96,"要確認")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F10" s="38" t="n">
         <x:f>SUM(B10:E10)</x:f>
@@ -1660,7 +1690,7 @@
       </x:c>
       <x:c r="I13"/>
     </x:row>
-    <x:row r="14" ht="31" customHeight="1">
+    <x:row r="14" ht="72" customHeight="1">
       <x:c r="A14" s="35" t="str">
         <x:v>AI添削</x:v>
       </x:c>
@@ -1689,7 +1719,7 @@
         <x:v>0.2222222222222222</x:v>
       </x:c>
       <x:c r="H14" s="43" t="str">
-        <x:v>Claude Edge Functionへ段階別添削指示・出力検証・利用量記録を接続</x:v>
+        <x:v>認証済みE2Eで実Claude問題生成・再利用・添削・履歴復元・実測費用を確認</x:v>
       </x:c>
       <x:c r="I14"/>
     </x:row>
@@ -1835,7 +1865,7 @@
       </x:c>
       <x:c r="C19" s="38" t="n">
         <x:f>COUNTIFS('実装タスク'!$C$5:$C$96,$A19,'実装タスク'!$F$5:$F$96,"進行中")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D19" s="38" t="n">
         <x:f>COUNTIFS('実装タスク'!$C$5:$C$96,$A19,'実装タスク'!$F$5:$F$96,"未着手")</x:f>
@@ -1843,7 +1873,7 @@
       </x:c>
       <x:c r="E19" s="38" t="n">
         <x:f>COUNTIFS('実装タスク'!$C$5:$C$96,$A19,'実装タスク'!$F$5:$F$96,"要確認")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F19" s="38" t="n">
         <x:f>SUM(B19:E19)</x:f>
@@ -1880,46 +1910,46 @@
       <x:c r="H21"/>
       <x:c r="I21"/>
     </x:row>
-    <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="193" t="str">
-        <x:v>現在地: STEP 1を5問、STEP 2・3を各3問のセット形式として、出題・入力・Claude一括採点・修正再提出・履歴・重複回避・旧未提出問題の更新まで実装済み。到達済み段階の選択は、別段階に未提出課題があっても許可し、元の段階へ戻ると課題を再開する。次は実アカウントでSTEP 1〜3の一部不正解と全問合格、段階往復を試し、Claude品質・DB保存・実測トークンを確認する。</x:v>
-      </x:c>
-      <x:c r="B22" s="193" t="str"/>
-      <x:c r="C22" s="193" t="str"/>
-      <x:c r="D22" s="193" t="str"/>
-      <x:c r="E22" s="193" t="str"/>
-      <x:c r="F22" s="193" t="str"/>
-      <x:c r="G22" s="193" t="str"/>
-      <x:c r="H22" s="193" t="str"/>
-      <x:c r="I22" s="193" t="str"/>
+    <x:row r="22" ht="100" customHeight="1">
+      <x:c r="A22" s="234" t="str">
+        <x:v>現在地: STEP 2で要修正後に合格すると、解説を表示せずSTEP 3へ進む不具合を修正した。原因は、提出保存で次段階が解放された直後に認証・DB状態の再読込が割り込み、未確認の提出結果より現在問題への自動遷移が優先される競合だった。全段階共通で、結果表示待ちを学習者が「解答を修正する」または「次の問題へ」を押すまで保持する。解説は1〜5件を必須とし、画面とDBの両方で0件を拒否する。全18ファイル190テスト、型検査、製品ビルドが成功。Supabase migration適用済み。Cloudflare Version 21a2dec9-ff4e-42a6-b376-a1e8f1e6d6bcへ公開し、トップ・課題一覧HTTP 200を確認。次は公開版でSTEP 2の要修正→再提出合格、一発合格、進級テスト合否の全経路で、解説確認後にのみ次へ進むことを確認する。最終テストでは問題生成・審査・修正・添削の暫定AI上限を所有者へ必ず確認する。</x:v>
+      </x:c>
+      <x:c r="B22" s="234" t="str"/>
+      <x:c r="C22" s="234" t="str"/>
+      <x:c r="D22" s="234" t="str"/>
+      <x:c r="E22" s="234" t="str"/>
+      <x:c r="F22" s="234" t="str"/>
+      <x:c r="G22" s="234" t="str"/>
+      <x:c r="H22" s="234" t="str"/>
+      <x:c r="I22" s="234" t="str"/>
       <x:c r="J22" s="46"/>
     </x:row>
-    <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="195" t="str">
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="235" t="str">
         <x:v>進捗は作業単位の更新履歴で管理します。開発者の日次活動と作業時間は記録しません。学習者向け活動グリッドはアプリ機能として維持します。</x:v>
       </x:c>
-      <x:c r="B23" s="195" t="str"/>
-      <x:c r="C23" s="195" t="str"/>
-      <x:c r="D23" s="195" t="str"/>
-      <x:c r="E23" s="195" t="str"/>
-      <x:c r="F23" s="195" t="str"/>
-      <x:c r="G23" s="195" t="str"/>
-      <x:c r="H23" s="195" t="str"/>
-      <x:c r="I23" s="195" t="str"/>
+      <x:c r="B23" s="235" t="str"/>
+      <x:c r="C23" s="235" t="str"/>
+      <x:c r="D23" s="235" t="str"/>
+      <x:c r="E23" s="235" t="str"/>
+      <x:c r="F23" s="235" t="str"/>
+      <x:c r="G23" s="235" t="str"/>
+      <x:c r="H23" s="235" t="str"/>
+      <x:c r="I23" s="235" t="str"/>
       <x:c r="J23" s="106"/>
     </x:row>
-    <x:row r="24" ht="22" customHeight="1">
-      <x:c r="A24" s="198" t="str">
-        <x:v>最終更新日: 2026-09-06　｜　進捗の正本: このファイル</x:v>
-      </x:c>
-      <x:c r="B24" s="198" t="str"/>
-      <x:c r="C24" s="198" t="str"/>
-      <x:c r="D24" s="198" t="str"/>
-      <x:c r="E24" s="198" t="str"/>
-      <x:c r="F24" s="198" t="str"/>
-      <x:c r="G24" s="198" t="str"/>
-      <x:c r="H24" s="198" t="str"/>
-      <x:c r="I24" s="198" t="str"/>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="236" t="str">
+        <x:v>最終更新日: 2026-09-15　｜　進捗の正本: このファイル</x:v>
+      </x:c>
+      <x:c r="B24" s="236" t="str"/>
+      <x:c r="C24" s="236" t="str"/>
+      <x:c r="D24" s="236" t="str"/>
+      <x:c r="E24" s="236" t="str"/>
+      <x:c r="F24" s="236" t="str"/>
+      <x:c r="G24" s="236" t="str"/>
+      <x:c r="H24" s="236" t="str"/>
+      <x:c r="I24" s="236" t="str"/>
       <x:c r="J24" s="47"/>
     </x:row>
   </x:sheetData>
@@ -2465,19 +2495,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H15" s="84" t="str">
-        <x:v>ホーム画面の学習開始導線を「学習を始める」一つに統一。メインナビゲーションの「進捗」を、設定画面も含むことが伝わる「進捗・設定」に変更。</x:v>
+        <x:v>ホーム・課題・履歴・進捗の導線を整理。課題トップの「復習する」「学習に戻る」は、段階変更を保存した直後に対象段階の未提出問題または次の問題へ直接移動する。一度最上部へ戻って「取り組む」を押す操作を廃止した。</x:v>
       </x:c>
       <x:c r="I15" s="84" t="str">
-        <x:v>ホーム画面と「進捗・設定」画面の導線を認証済みE2Eで確認する。</x:v>
+        <x:v>公開版で下部にある完了済み段階と最高到達段階を選び、1回のクリックで正しい問題画面へ移ることを確認する。</x:v>
       </x:c>
       <x:c r="J15" s="77" t="str">
         <x:v>主要画面へURLで移動できる</x:v>
       </x:c>
       <x:c r="K15" s="77" t="str">
-        <x:v>web/src/routes/ / web/src/app.css</x:v>
+        <x:v>web/src/routes/tasks/+page.svelte / docs/architecture.md</x:v>
       </x:c>
       <x:c r="L15" s="88" t="n">
-        <x:v>46270</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="125" customHeight="1">
@@ -2542,10 +2572,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H17" s="84" t="str">
-        <x:v>STEP 1の修正画面で正解済みを保持してロック。不正解だけ修正でき、再読み込み時も提出結果と下書きから復元する。</x:v>
+        <x:v>要修正の再表示では、正式添削結果に保存された通常版またはやさしい版の一種類だけを入力欄の直前へ復元する。追加生成された別解説の読込と保存は廃止した。正解済み解答と下書きの復元は維持。</x:v>
       </x:c>
       <x:c r="I17" s="84" t="str">
-        <x:v>公開版の実アカウントでも再読み込みと修正途中の復元を確認する。</x:v>
+        <x:v>実アカウントで設定OFF/ONそれぞれの要修正→画面再読込→再提出を行い、同じ一種類の解説と下書き・正解済み解答が保持されることを確認する。</x:v>
       </x:c>
       <x:c r="J17" s="77" t="str">
         <x:v>再読込後も下書きが復元される</x:v>
@@ -2554,10 +2584,10 @@
         <x:v>web/src/lib/features/learning/learning-service.ts / web/src/lib/features/learning/save-queue.ts / web/src/routes/tasks/</x:v>
       </x:c>
       <x:c r="L17" s="232" t="n">
-        <x:v>46270</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="150" customHeight="1">
+        <x:v>46274</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="155" customHeight="1">
       <x:c r="A18" s="77" t="str">
         <x:v>APP-007</x:v>
       </x:c>
@@ -2580,22 +2610,22 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H18" s="84" t="str">
-        <x:v>STEP 1を5問、STEP 2・3を各3問のセット提出へ統一。到達済み段階の選択時、別段階に未提出課題があっても移動できるようにし、未提出課題は削除せず該当段階へ戻ったときに再開する。</x:v>
+        <x:v>正式提出・添削・書き直しに加え、提出成功後の結果表示待ち状態を同一タブへ保持する。要修正後の合格、一発合格、進級テストの合否は、認証・DB状態の再読込が起きても結果と解説を復元し、学習者が「解答を修正する」または「次の問題へ」を選ぶまで自動遷移しない。</x:v>
       </x:c>
       <x:c r="I18" s="84" t="str">
-        <x:v>利用者画面でSTEP 1（Haiku）、STEP 2・3（Sonnet）の合格・一部不正解・修正再提出に加え、未提出課題を残した段階往復を確認する。</x:v>
+        <x:v>認証済み公開画面でSTEP 2の要修正→修正→合格を行い、3問すべての解説を確認してから「次の問題へ」でSTEP 3へ進むことを確認する。あわせて一発合格と進級テストの合否でも同じ結果表示を確認する。</x:v>
       </x:c>
       <x:c r="J18" s="77" t="str">
         <x:v>提出状態と結果が永続化される</x:v>
       </x:c>
       <x:c r="K18" s="77" t="str">
-        <x:v>web/src/routes/tasks/[taskId]/ / web/src/lib/features/learning/progression.ts</x:v>
+        <x:v>web/src/routes/tasks/[taskId]/+page.svelte / web/src/lib/features/learning/submission-workflow.ts / progression.ts</x:v>
       </x:c>
       <x:c r="L18" s="232" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="150" customHeight="1">
+        <x:v>46280</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="155" customHeight="1">
       <x:c r="A19" s="77" t="str">
         <x:v>APP-008</x:v>
       </x:c>
@@ -2618,10 +2648,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H19" s="84" t="str">
-        <x:v>提出履歴でSTEP 1〜3の全問題について、指示・問題文・解答・正誤・解説を対応表示。到達済み段階へ戻っても、各段階の未提出課題と提出履歴を保持する。</x:v>
+        <x:v>提出履歴と進捗を表示。段階状態を「完了」「復習中」「学習中」「未完了」に分け、復習から最高到達段階へ戻る操作を「学習に戻る」と表示する。復習によって先の段階を閉じない。</x:v>
       </x:c>
       <x:c r="I19" s="84" t="str">
-        <x:v>認証済みE2Eで3問セットの履歴と、修正後も正解済み答案が保持されること、段階往復後に未提出課題を再開できることを確認する。</x:v>
+        <x:v>認証済みE2Eで全段階の進級、ページ移動、復習、最高到達段階への復帰を確認する。</x:v>
       </x:c>
       <x:c r="J19" s="77" t="str">
         <x:v>ユーザー自身の履歴だけが表示される</x:v>
@@ -2630,7 +2660,7 @@
         <x:v>web/src/routes/ / web/src/lib/features/learning/learning-service.ts</x:v>
       </x:c>
       <x:c r="L19" s="232" t="n">
-        <x:v>46271</x:v>
+        <x:v>46272</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -2852,19 +2882,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H25" s="84" t="str">
-        <x:v>段階1〜13の各10問、合計130問をcurriculum.jsonへ生成。ID・段階・話題重複を検証</x:v>
+        <x:v>STEP 1〜3は各10セットを維持し、STEP 4〜14は大学入試小論文を想定した78の共通論点へ拡張。全858題で設問・主張・理由・具体例・反対意見・結論の向きを段階間で統一した。カリキュラム全体は888課題。</x:v>
       </x:c>
       <x:c r="I25" s="84" t="str">
-        <x:v>練習テーマ追加時にpractice-bankと検証テストを同時更新</x:v>
+        <x:v>代表論点を実画面で確認し、入試課題としての難易度・語彙・論点の偏りを継続監査する。</x:v>
       </x:c>
       <x:c r="J25" s="77" t="str">
         <x:v>生成結果が検証を通る</x:v>
       </x:c>
       <x:c r="K25" s="77" t="str">
-        <x:v>web/scripts/practice-bank.ts / web/src/lib/data/curriculum.json</x:v>
+        <x:v>web/src/lib/data/essay-topic-bank.ts / web/scripts/practice-bank.ts / web/src/lib/data/curriculum.json</x:v>
       </x:c>
       <x:c r="L25" s="88" t="n">
-        <x:v>46259</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
@@ -2872,7 +2902,6 @@
         <x:v>CUR-006</x:v>
       </x:c>
       <x:c r="B26" s="70" t="str">
-        <x:f>IF(F26="完了","☑","☐")</x:f>
         <x:v>☑</x:v>
       </x:c>
       <x:c r="C26" s="62" t="str">
@@ -2891,19 +2920,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H26" s="84" t="str">
-        <x:v>130問を現在段階の1問ずつへ接続し、全問使用後も直前と同じ問題を避ける</x:v>
+        <x:v>STEP 1は5問×10セット、STEP 2・3は3問×10セットの個別設計を維持。STEP 4〜14へ78論点を接続し、設定に応じて固定論点または学習者の自由テーマを使う構成へ更新した。</x:v>
       </x:c>
       <x:c r="I26" s="84" t="str">
-        <x:v>本番問題追加時に話題キーと教育内容をレビュー</x:v>
+        <x:v>公開画面でSTEP 4・7・9・14の固定論点と自由テーマ問題を解き、指示の理解しやすさと自然な別解のClaude判定を確認する。</x:v>
       </x:c>
       <x:c r="J26" s="77" t="str">
         <x:v>Excel由来の課題が画面に出る</x:v>
       </x:c>
       <x:c r="K26" s="77" t="str">
-        <x:v>web/src/lib/data/curriculum.ts / web/src/lib/features/learning/progression.ts / web/src/routes/tasks/</x:v>
+        <x:v>web/src/lib/data/essay-topic-bank.ts / web/src/lib/features/learning/problem-generator.ts / web/src/lib/data/curriculum.test.ts</x:v>
       </x:c>
       <x:c r="L26" s="88" t="n">
-        <x:v>46259</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
@@ -3310,19 +3339,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H37" s="84" t="str">
-        <x:v>実DBで不正解→同じセットへ再提出→合格の回帰テスト成功。冪等性・進級テスト・ユーザー分離も成功。テストデータはロールバック。</x:v>
+        <x:v>実DBのRLS・冪等性・進級テスト・ユーザー分離を検証済み。さらに、正式提出にはSTEP 1〜3の複数問とSTEP 4〜14の単問に対応する1〜5件の学習者向け解説を必須とし、解説0件の不完全な結果を保存前に拒否するDB制約をオンライン適用した。</x:v>
       </x:c>
       <x:c r="I37" s="84" t="str">
-        <x:v>Claude接続後も同じ回帰テストを継続する。</x:v>
+        <x:v>Claude異常出力として解説0件・6件以上を返すケースと、STEP 1の5件・STEP 2/3の3件・STEP 4以降の1件を認証済みE2Eで確認する。</x:v>
       </x:c>
       <x:c r="J37" s="77" t="str">
         <x:v>許可・拒否ケースが全て成功</x:v>
       </x:c>
       <x:c r="K37" s="77" t="str">
-        <x:v>supabase/tests/learner_data_rls.sql</x:v>
+        <x:v>supabase/migrations/202609150001_require_feedback_comments.sql / supabase/tests/learner_data_rls.sql</x:v>
       </x:c>
       <x:c r="L37" s="232" t="n">
-        <x:v>46270</x:v>
+        <x:v>46280</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="110" customHeight="1">
@@ -3348,19 +3377,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H38" s="84" t="str">
-        <x:v>適用後の整合性11項目はすべて不整合0件。既存データを削除せず更新。</x:v>
+        <x:v>下書き・提出・添削・進捗・解説難易度に加え、論点選択方式と自由設定テーマをlearning_progressへ保存。DB制約でランダム／自由設定、1〜3件、各20文字以内、空白・重複を検査し、本人だけに更新を許可した。</x:v>
       </x:c>
       <x:c r="I38" s="84" t="str">
-        <x:v>問題生成・添削の接続後も監査を実行する。</x:v>
+        <x:v>実アカウントで設定保存、再読込、別端末同期、別ユーザー分離を確認する。</x:v>
       </x:c>
       <x:c r="J38" s="77" t="str">
         <x:v>再読込後もデータが維持される</x:v>
       </x:c>
       <x:c r="K38" s="77" t="str">
-        <x:v>supabase/migrations/202608210001_initial_schema.sql / web/src/lib/features/learning/learning-service.ts</x:v>
+        <x:v>supabase/migrations/202609100001_topic_preferences_and_expanded_bank.sql / web/src/lib/features/learning/learning-service.ts</x:v>
       </x:c>
       <x:c r="L38" s="232" t="n">
-        <x:v>46270</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="48" customHeight="1">
@@ -3497,16 +3526,16 @@
         <x:v>feedback Edge Functionを実装する</x:v>
       </x:c>
       <x:c r="F42" s="83" t="str">
-        <x:v>要確認</x:v>
+        <x:v>進行中</x:v>
       </x:c>
       <x:c r="G42" s="83" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H42" s="84" t="str">
-        <x:v>feedback Edge FunctionをSTEP 1の5問とSTEP 2・3の3問一括採点へ拡張。段階別カテゴリ・件数・問題ID・全問正解判定を検証し、Supabaseへ配備。</x:v>
+        <x:v>feedback Edge Functionを更新し、languageStatus（日本語表現上の状態）とdecision（当該STEPの達成判定）を分離した。cleanかつreviseを正当な組み合わせとして許可し、revision_requiredかつpassは引き続き拒否する。Claudeへの指示、回帰テスト、検証失敗時の実使用量記録も追加し、Supabaseへ配備済み。</x:v>
       </x:c>
       <x:c r="I42" s="84" t="str">
-        <x:v>利用者画面からSTEP 1〜3を提出し、モデル別の判定・正式保存・進捗更新を確認する。</x:v>
+        <x:v>オンライン環境で同じ答案を再提出し、cleanかつreviseの判定が要修正結果として保存・表示されることを確認する。その後、STEP 2・3の自然な別解も確認する。</x:v>
       </x:c>
       <x:c r="J42" s="77" t="str">
         <x:v>正常・異常ケースがテストを通る</x:v>
@@ -3515,10 +3544,10 @@
         <x:v>supabase/functions/feedback/</x:v>
       </x:c>
       <x:c r="L42" s="232" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="140" customHeight="1">
+        <x:v>46275</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="145" customHeight="1">
       <x:c r="A43" s="77" t="str">
         <x:v>AI-004</x:v>
       </x:c>
@@ -3541,19 +3570,19 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H43" s="84" t="str">
-        <x:v>Anthropic呼出を共通化し、STEP 1・4はHaiku 4.5、STEP 2・3とSTEP 5〜14はSonnet 4.6を使用。STEP 3の論理構成3問化に合わせ、旧Haiku設定からSonnetへ変更。</x:v>
+        <x:v>Anthropic呼出を共通化。添削のHaiku 4.5・Sonnet 4.6とは別に、問題生成を標準Sonnet 5としてproblem-generation Edge Functionへ接続し、Supabaseへ配備した。モデルIDはサーバー環境変数で変更できる。</x:v>
       </x:c>
       <x:c r="I43" s="84" t="str">
-        <x:v>Claude問題生成を追加する際に同じ呼出境界を再利用し、プロバイダー差替え契約を完成する。</x:v>
+        <x:v>実ユーザーの新規問題生成でSonnet 5の正常応答、応答時間、教育品質を確認する。将来ほかの提供元を採用する場合は同じ呼出境界へ実装する。</x:v>
       </x:c>
       <x:c r="J43" s="77" t="str">
         <x:v>モックとClaudeを設定で切替可能</x:v>
       </x:c>
       <x:c r="K43" s="77" t="str">
-        <x:v>supabase/functions/_shared/</x:v>
+        <x:v>supabase/functions/_shared/claude.ts / runtime.ts / problem-generation.ts</x:v>
       </x:c>
       <x:c r="L43" s="232" t="n">
-        <x:v>46271</x:v>
+        <x:v>46274</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="140" customHeight="1">
@@ -3579,10 +3608,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H44" s="84" t="str">
-        <x:v>STEP 2は情報関係・明確さ・情報選択、STEP 3は順序・不足説明・流れ修正を採点する段階別指示へ更新。正解例との文字列一致ではなく自然な言い換えを許容する。</x:v>
+        <x:v>解説難易度の条件は通常feedbackプロンプト内だけで制御する。結果後の追加言い換え用プロンプト・契約・クライアント呼出を削除し、設定OFF/ONで別の説明を二重保存しない構成にした。</x:v>
       </x:c>
       <x:c r="I44" s="84" t="str">
-        <x:v>実答案で許容範囲と助言の分かりやすさを確認し、使用プロンプト版の保存を追加する。</x:v>
+        <x:v>実答案で通常版とやさしい版を比較し、小学校高学年〜中学生を目安とした読みやすさと採点基準不変を確認する。使用プロンプト版の保存も追加する。</x:v>
       </x:c>
       <x:c r="J44" s="77" t="str">
         <x:v>結果に使用バージョンが保存される</x:v>
@@ -3591,10 +3620,10 @@
         <x:v>web/src/lib/features/learning/feedback.ts / learning-design.ts / docs/architecture.md</x:v>
       </x:c>
       <x:c r="L44" s="232" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="140" customHeight="1">
+        <x:v>46274</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="145" customHeight="1">
       <x:c r="A45" s="77" t="str">
         <x:v>AI-006</x:v>
       </x:c>
@@ -3617,22 +3646,22 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H45" s="84" t="str">
-        <x:v>STEP 1〜3の問題セット用構造化出力を共通化。入力と同数の結果、問題ID、合否・言語状態の整合をEdge Functionで再検証し、不正出力は保存しない。</x:v>
+        <x:v>添削結果のJSON Schema検証とサーバー再検証を実装。languageStatusは表現上の状態、decisionは段階目標の達成判定として扱い、cleanかつreviseを許可する。合格なのに重大な未達、revision_requiredなのに合格、要修正なのに全技能達成、実回答を未回答とする結果は拒否する。</x:v>
       </x:c>
       <x:c r="I45" s="84" t="str">
-        <x:v>STEP 2・3の実Claude応答で全問結果と履歴スナップショットを確認する。</x:v>
+        <x:v>実アカウントでcleanかつrevise、minor_issueかつpass、revision_requiredかつreviseの代表ケースを確認する。破損出力を安全に拒否できることも認証済みE2Eへ追加する。</x:v>
       </x:c>
       <x:c r="J45" s="77" t="str">
         <x:v>破損出力を安全に拒否できる</x:v>
       </x:c>
       <x:c r="K45" s="77" t="str">
-        <x:v>supabase/functions/feedback/</x:v>
+        <x:v>supabase/functions/_shared/problem-generation-contract.ts / problem-generation-prompt.ts</x:v>
       </x:c>
       <x:c r="L45" s="232" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="130" customHeight="1">
+        <x:v>46275</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="145" customHeight="1">
       <x:c r="A46" s="77" t="str">
         <x:v>AI-007</x:v>
       </x:c>
@@ -3655,10 +3684,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H46" s="84" t="str">
-        <x:v>確定したClaudeエラーでは次の提出に新しいrequest_idを発行し、通信結果が不明な場合と処理中だけ同じIDを再利用するよう修正。失敗した提出は正式成績へ保存しない。</x:v>
+        <x:v>問題生成に認証、安定request_id、DB予約、暫定日次予算、検証失敗時1回だけ再生成、失敗記録、確認済みローカル問題への退避を実装。承認済み問題は再利用してClaude呼出と重複課金を避ける。</x:v>
       </x:c>
       <x:c r="I46" s="84" t="str">
-        <x:v>利用者画面でエラー後の再提出と、正常時の二重保存防止を確認する。</x:v>
+        <x:v>実環境で生成成功、再利用、予算超過、提供元障害の挙動を確認する。最終公開テスト時に問題生成・添削の暫定上限をサービス責任者へ必ず再確認する。</x:v>
       </x:c>
       <x:c r="J46" s="77" t="str">
         <x:v>障害時に安全なエラーを返す</x:v>
@@ -3667,7 +3696,7 @@
         <x:v>supabase/functions/feedback/</x:v>
       </x:c>
       <x:c r="L46" s="232" t="n">
-        <x:v>46271</x:v>
+        <x:v>46274</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
@@ -4215,7 +4244,7 @@
         <x:v>46268</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="140" customHeight="1">
+    <x:row r="61" ht="145" customHeight="1">
       <x:c r="A61" s="77" t="str">
         <x:v>OPS-002</x:v>
       </x:c>
@@ -4238,19 +4267,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H61" s="84" t="str">
-        <x:v>STEP 2・3の3問セット画面、旧未提出課題の安全な現行版更新、Claude一括採点を公開。Supabase migration・feedback Functionを適用し、Cloudflare Version 8f2c1e38-0980-40a4-a018-5e7dcabb8b62へ配備。</x:v>
+        <x:v>提出結果を必ず表示してから次へ進む修正をCloudflare検証環境へ公開。Supabaseには解説1〜5件を必須とするmigrationを適用。Cloudflare Version 21a2dec9-ff4e-42a6-b376-a1e8f1e6d6bc。トップと課題一覧はHTTP 200。</x:v>
       </x:c>
       <x:c r="I61" s="84" t="str">
-        <x:v>公開画面でSTEP 2・3の入力・提出・修正・履歴を確認する。</x:v>
+        <x:v>ブラウザを1回再読込して新版を取得し、STEP 2の要修正→修正→合格で解説を確認後、「次の問題へ」を押してSTEP 3へ進む。代表段階と進級テストでも同じ順序を確認する。</x:v>
       </x:c>
       <x:c r="J61" s="77" t="str">
         <x:v>検証URLで認証・保存・再読込・ユーザー分離・学習遷移が成功する</x:v>
       </x:c>
       <x:c r="K61" s="77" t="str">
-        <x:v>web/wrangler.jsonc / docs/cloudflare-staging.md</x:v>
+        <x:v>Cloudflare Workers / web/src/routes/tasks/[taskId]/+page.svelte</x:v>
       </x:c>
       <x:c r="L61" s="232" t="n">
-        <x:v>46271</x:v>
+        <x:v>46280</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
@@ -4409,7 +4438,7 @@
         <x:v>46258</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="140" customHeight="1">
+    <x:row r="66" ht="145" customHeight="1">
       <x:c r="A66" s="77" t="str">
         <x:v>QA-001</x:v>
       </x:c>
@@ -4432,19 +4461,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H66" s="84" t="str">
-        <x:v>STEP 1〜3のセット出題、ローテーション、Claude契約、修正再提出、履歴、旧問題更新を含む17ファイル122テストが成功。型検査0エラー・0警告、製品ビルド成功。公開STEP 2・3はHTTP 200。</x:v>
+        <x:v>次問をDBへ発行・再取得してから遷移する回帰検査を追加。進級テスト開始を含む関連66テストと、全18ファイル186テストが成功。型検査0エラー・0警告、製品ビルド成功。</x:v>
       </x:c>
       <x:c r="I66" s="84" t="str">
-        <x:v>認証済みの実画面E2EとClaude品質・実測トークン確認を追加する。</x:v>
+        <x:v>公開画面の実セッションで、訓練から進級テストへの境界と、進級テスト各問の連続遷移を確認する。</x:v>
       </x:c>
       <x:c r="J66" s="77" t="str">
         <x:v>主要ロジックのテストがCIで成功</x:v>
       </x:c>
       <x:c r="K66" s="77" t="str">
-        <x:v>web/src/**/*.test.ts / .github/workflows/verify.yml</x:v>
+        <x:v>web/src/lib/features/learning/ui-copy.test.ts / task-flow.test.ts / progression.test.ts / submission-workflow.test.ts</x:v>
       </x:c>
       <x:c r="L66" s="232" t="n">
-        <x:v>46271</x:v>
+        <x:v>46279</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
@@ -4861,19 +4890,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H77" t="str">
-        <x:v>14段階の出題へ再編。段階1は5領域から1問ずつ選ぶセット、段階7は役割判別・不要文削除・並べ替え・不足説明補完を組み合わせた問題へ更新</x:v>
+        <x:v>STEP 4〜14は78の固定論点から、履歴の使用回数・分野・類似度を考慮して未出題を優先する。自由設定では1〜3テーマを順に使い、テーマ固有IDで固定論点や別テーマとの混在を防ぐ。</x:v>
       </x:c>
       <x:c r="I77" t="str">
-        <x:v>Claude生成問題にも14段階の本文・ヒント分離と段階1の構造化5問形式を適用</x:v>
+        <x:v>実アカウントで固定論点の循環、自由テーマ切替、過去問題との重複回避を確認する。</x:v>
       </x:c>
       <x:c r="J77" t="str">
         <x:v>同じ段階で未出題が優先され、直前と同一問題が連続しない</x:v>
       </x:c>
       <x:c r="K77" t="str">
-        <x:v>web/scripts/practice-bank.ts / web/src/lib/features/learning/problem-generator.ts</x:v>
+        <x:v>web/src/lib/data/essay-topic-bank.ts / web/src/lib/features/learning/progression.ts / problem-generator.ts</x:v>
       </x:c>
       <x:c r="L77" s="55" t="n">
-        <x:v>46267</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -4900,19 +4929,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H78" t="str">
-        <x:v>通常トレーニング10回合格後、進級テストで累積3回合格すると進級。全課程を14段階へ拡張し、段階1は5問全問正解で1回合格する方式を実装</x:v>
+        <x:v>進級テスト開始直後の入力ロック修正に加え、提出結果より次段階の解放が先に反映された場合でも、未確認の合否・解説を飛ばさない遷移境界を全段階へ共通実装した。次問発行は結果画面の「次の問題へ」を押した後だけ行う。</x:v>
       </x:c>
       <x:c r="I78" t="str">
-        <x:v>認証済みブラウザE2Eで段階1の5問セット、段階7、段階14修了を確認</x:v>
+        <x:v>認証済み公開画面で、STEP 2の再提出合格と通常合格、進級テスト合否をそれぞれ確認し、解説表示後の操作だけで次問・次段階へ進むことを確認する。</x:v>
       </x:c>
       <x:c r="J78" t="str">
         <x:v>通常トレーニングの合格数が減らず、進級テストで不合格を挟んでも規定合格数で次段階へ進む</x:v>
       </x:c>
       <x:c r="K78" t="str">
-        <x:v>web/src/lib/features/learning/progression.ts / web/src/routes/tasks/ / web/src/routes/progress/</x:v>
+        <x:v>web/src/routes/tasks/[taskId]/+page.svelte / web/src/lib/features/learning/ui-copy.test.ts</x:v>
       </x:c>
       <x:c r="L78" s="55" t="n">
-        <x:v>46267</x:v>
+        <x:v>46280</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -4976,19 +5005,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H80" s="211" t="str">
-        <x:v>隔離Chromiumの1100px・390px幅で要修正／合格のスクロール位置、解答保持、再読み込み、再提出、履歴の不正解強調を確認。JS例外なし。</x:v>
+        <x:v>提出結果を未確認のまま自動遷移しない共通状態を追加。古い提出IDは30分で失効する一方、保存済み結果の表示待ちは学習者の操作まで保持する。空の解説を拒否し、最大5問の解説を受け入れる単体・画面・SQL契約テストを追加した。全18ファイル190テスト、型検査、製品ビルドが成功。</x:v>
       </x:c>
       <x:c r="I80" s="211" t="str">
-        <x:v>認証済み公開画面で確認を継続。DBと合格数計算は今回変更なし。</x:v>
+        <x:v>公開版でSTEP 2の要修正→再提出合格、STEP 1の5問合格、STEP 4以降の単問合格、進級テスト不合格・合格を操作し、すべて解説表示後にのみ遷移することを確認する。</x:v>
       </x:c>
       <x:c r="J80" s="211" t="str">
         <x:v>ローカル・実DB・E2Eの主要境界ケースが成功する</x:v>
       </x:c>
       <x:c r="K80" s="211" t="str">
-        <x:v>web/src/**/*.test.ts / supabase/tests/learner_data_rls.sql</x:v>
+        <x:v>web/src/lib/features/learning/submission-workflow.ts / learning-service.ts / ui-copy.test.ts / sql-contract.test.ts</x:v>
       </x:c>
       <x:c r="L80" s="213" t="n">
-        <x:v>46270</x:v>
+        <x:v>46280</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="140" customHeight="1">
@@ -5008,25 +5037,25 @@
         <x:v>問題数を固定せず段階別特徴署名で異なる傾向を選ぶ</x:v>
       </x:c>
       <x:c r="F81" s="211" t="str">
-        <x:v>進行中</x:v>
+        <x:v>要確認</x:v>
       </x:c>
       <x:c r="G81" s="211" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H81" s="211" t="str">
-        <x:v>STEP 2・3は各3領域の問題を組み合わせ、27セットを重複なく選択。セット内容を問題識別値に含める。STEP 1は5問セットを維持。</x:v>
+        <x:v>段階別特徴署名による類似回避に、78論点と自由設定テーマを追加。ランダム利用者には自由テーマ由来の共有問題を出さず、自由設定では一致するテーマ固有IDの問題だけを再利用する。</x:v>
       </x:c>
       <x:c r="I81" s="211" t="str">
-        <x:v>27セット消化前にClaude問題生成・検証・問題バンク補充を実装する。</x:v>
+        <x:v>認証済みE2Eで自由テーマのClaude生成・同テーマ再利用・ランダム設定への非混入・履歴復元を確認する。</x:v>
       </x:c>
       <x:c r="J81" s="211" t="str">
         <x:v>履歴・技能統計から説明可能に次の訓練目標を選び、同一傾向を避けられる</x:v>
       </x:c>
       <x:c r="K81" s="211" t="str">
-        <x:v>web/src/lib/features/learning/problem-generator.ts / progression.ts / docs/architecture.md</x:v>
+        <x:v>web/src/lib/features/learning/topic-preferences.ts / progression.ts / problem-generator.ts / docs/architecture.md</x:v>
       </x:c>
       <x:c r="L81" s="213" t="n">
-        <x:v>46271</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -5106,42 +5135,42 @@
         <x:v>46260</x:v>
       </x:c>
     </x:row>
-    <x:row r="84">
-      <x:c r="A84" t="str">
+    <x:row r="84" ht="145" customHeight="1">
+      <x:c r="A84" s="211" t="str">
         <x:v>QA-009</x:v>
       </x:c>
-      <x:c r="B84" t="str">
+      <x:c r="B84" s="211" t="str">
         <x:v>☐</x:v>
       </x:c>
-      <x:c r="C84" t="str">
+      <x:c r="C84" s="211" t="str">
         <x:v>テスト・運用・法務</x:v>
       </x:c>
-      <x:c r="D84" t="str">
+      <x:c r="D84" s="211" t="str">
         <x:v>動的出題・段階往復</x:v>
       </x:c>
-      <x:c r="E84" t="str">
+      <x:c r="E84" s="211" t="str">
         <x:v>問題生成、特徴検証、旧データ移行、段階往復を回帰テストする</x:v>
       </x:c>
-      <x:c r="F84" t="str">
+      <x:c r="F84" s="211" t="str">
         <x:v>進行中</x:v>
       </x:c>
-      <x:c r="G84" t="str">
+      <x:c r="G84" s="211" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="H84" t="str">
-        <x:v>67単体テスト、型検査、製品ビルド、実DBの14段階・段階1一回完了・累積合格式進級のRLS/RPCテストが成功</x:v>
-      </x:c>
-      <x:c r="I84" t="str">
-        <x:v>認証済みE2EとClaude生成後の多様性・履歴保持を追加</x:v>
-      </x:c>
-      <x:c r="J84" t="str">
+      <x:c r="H84" s="211" t="str">
+        <x:v>固定78論点と自由テーマについて、特徴署名、テーマ固有ID、問題URL復元、STEP 4未満の拒否、20文字上限、固定問題との分離を回帰テストへ追加。全166テストと製品ビルドが成功。</x:v>
+      </x:c>
+      <x:c r="I84" s="211" t="str">
+        <x:v>公開環境で設定変更前後の未提出問題維持と、次問への反映を認証済みE2Eで確認する。</x:v>
+      </x:c>
+      <x:c r="J84" s="211" t="str">
         <x:v>ローカル・実DB・E2Eで適応出題、履歴、段階状態、二重計上防止が一致する</x:v>
       </x:c>
-      <x:c r="K84" t="str">
-        <x:v>web/src/**/*.test.ts / supabase/tests/learner_data_rls.sql</x:v>
-      </x:c>
-      <x:c r="L84" s="55" t="n">
-        <x:v>46267</x:v>
+      <x:c r="K84" s="211" t="str">
+        <x:v>web/src/lib/features/learning/problem-generator.test.ts / progression.test.ts / sql-contract.test.ts</x:v>
+      </x:c>
+      <x:c r="L84" s="213" t="n">
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
@@ -5167,10 +5196,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H85" s="211" t="str">
-        <x:v>全14段階を、文の基礎→一文修正→文間関係→意見と理由→段落分析・構築→要約・資料・反対意見→構成メモ→小論文へ再設計。段階1と7の詳細仕様を確定</x:v>
+        <x:v>全14段階の技能順序を維持しつつ、STEP 1〜3の固定10セットを個別設計。STEP 7・9・10・12・14は、素材の役割、残す・除く情報、反対意見への応答、資料と自分の意見の区別を課題文へ明記した。</x:v>
       </x:c>
       <x:c r="I85" s="211" t="str">
-        <x:v>実利用ログから各段階の負荷、標準合格数、段階1の問題パターンを定期レビュー</x:v>
+        <x:v>実利用結果をもとに各セットの負荷、語彙、指示の理解しやすさ、標準合格数を再評価する。</x:v>
       </x:c>
       <x:c r="J85" s="211" t="str">
         <x:v>各段階の訓練目標・必須要素・特徴がコードと設計書で一致する</x:v>
@@ -5179,7 +5208,7 @@
         <x:v>docs/architecture.md / web/src/lib/features/learning/learning-design.ts / web/scripts/convert-curriculum.ts</x:v>
       </x:c>
       <x:c r="L85" s="55" t="n">
-        <x:v>46267</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
@@ -5220,7 +5249,7 @@
         <x:v>46260</x:v>
       </x:c>
     </x:row>
-    <x:row r="87" ht="125" customHeight="1">
+    <x:row r="87" ht="145" customHeight="1">
       <x:c r="A87" s="211" t="str">
         <x:v>DB-010</x:v>
       </x:c>
@@ -5243,60 +5272,60 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H87" s="211" t="str">
-        <x:v>AI予約テーブルとサービス専用RPCをmigrationで適用。ブラウザのsubmit_mock実行権限を削除し、利用量と正式提出を同一トランザクションで保存。</x:v>
+        <x:v>共有問題バンクへtrial状態を追加し、生成時の独立品質審査、問題別試行回数、最終処理理由を保存する。合格した共通テーマ問題だけapprovedへ昇格し、自由テーマはprivate_verifiedとして共有しない。5回目の要修正ではrejectedへ移し、履歴を閉じて模範解答を返す。サービスロール専用表とRLSをオンラインDBで検証済み。</x:v>
       </x:c>
       <x:c r="I87" s="211" t="str">
-        <x:v>問題生成Edge Functionから問題バンクへ安全に登録する専用RPCを追加する。</x:v>
+        <x:v>実Claude生成E2E後もtrial隔離、5回終了、共通テーマ合格時だけの共有昇格、自由テーマ非共有を定期回帰テストする。</x:v>
       </x:c>
       <x:c r="J87" s="211" t="str">
         <x:v>本人の技能統計が隔離され、承認済み問題を安全に共有・再利用できる</x:v>
       </x:c>
       <x:c r="K87" s="211" t="str">
-        <x:v>supabase/migrations/202608210001_initial_schema.sql / supabase/tests/</x:v>
+        <x:v>supabase/migrations/202609110003_generated_problem_quality_lifecycle.sql / supabase/tests/generated_problem_quality_lifecycle.sql / web/src/lib/types/database.ts</x:v>
       </x:c>
       <x:c r="L87" s="213" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="48" customHeight="1">
-      <x:c r="A88" t="str">
+        <x:v>46276</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="145" customHeight="1">
+      <x:c r="A88" s="211" t="str">
         <x:v>AI-008</x:v>
       </x:c>
-      <x:c r="B88" t="str">
+      <x:c r="B88" s="211" t="str">
         <x:v>☐</x:v>
       </x:c>
-      <x:c r="C88" t="str">
+      <x:c r="C88" s="211" t="str">
         <x:v>AI添削</x:v>
       </x:c>
-      <x:c r="D88" t="str">
+      <x:c r="D88" s="211" t="str">
         <x:v>問題生成</x:v>
       </x:c>
-      <x:c r="E88" t="str">
+      <x:c r="E88" s="211" t="str">
         <x:v>Claudeで自然な問題文を生成・検証し問題バンクへ蓄積する</x:v>
       </x:c>
-      <x:c r="F88" t="str">
-        <x:v>進行中</x:v>
-      </x:c>
-      <x:c r="G88" t="str">
+      <x:c r="F88" s="211" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="G88" s="211" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H88" s="211" t="str">
-        <x:v>短いProblemSpecification、段階条件検証、n-gram類似検査、問題バンク優先、在庫不足時だけAI生成する契約とフォールバックを実装</x:v>
+        <x:v>Claudeのinformation_selection生成指示と構造検査を簡潔な自然文へ対応。問題文は意見・目的・方針・話題と番号付き材料を示し、2文以内で組み合わせ方と言い換え可を伝える。入力契約は短い有効表現を許可しつつ、使う材料と除く材料が不明な問題は引き続き拒否する。生成プロンプト版はproblem-generation-v5。</x:v>
       </x:c>
       <x:c r="I88" s="211" t="str">
-        <x:v>Claude Edge Functionの構造化出力・1回再試行・問題バンク登録を実装</x:v>
+        <x:v>認証済みテスト利用者でSTEP 2の固定10セット後にClaude生成を実行し、簡潔さと採点条件の一致を確認する。</x:v>
       </x:c>
       <x:c r="J88" s="211" t="str">
         <x:v>不正・重複・条件逸脱問題を発行せず、生成コストと版を記録できる</x:v>
       </x:c>
       <x:c r="K88" s="211" t="str">
-        <x:v>web/src/lib/features/learning/problem-generator.ts / ai-budget.ts / docs/architecture.md</x:v>
-      </x:c>
-      <x:c r="L88" s="92" t="n">
-        <x:v>46260</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="140" customHeight="1">
+        <x:v>supabase/functions/_shared/problem-generation-prompt.ts / problem-generation-contract.ts / problem-quality-prompt.ts</x:v>
+      </x:c>
+      <x:c r="L88" s="213" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="145" customHeight="1">
       <x:c r="A89" s="211" t="str">
         <x:v>QA-010</x:v>
       </x:c>
@@ -5313,25 +5342,25 @@
         <x:v>苦手反映・多様性・生成検証・フォールバックを検証する</x:v>
       </x:c>
       <x:c r="F89" s="211" t="str">
-        <x:v>進行中</x:v>
+        <x:v>要確認</x:v>
       </x:c>
       <x:c r="G89" s="211" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H89" s="211" t="str">
-        <x:v>STEP 2・3の件数・カテゴリ・問題ハッシュ・27セット重複回避を含む122単体テストが成功。Supabase migration履歴一致、公開STEP 2・3 HTTP 200。</x:v>
+        <x:v>固定問題消費後のtrial問題IDから試用識別子が失われ、DBの発行済み問題と一致しないため入力がロックされる原因を特定・修正。STEP 1〜14、選択式・記述式、自由テーマ、QA識別子を同じ復元処理で検査し、既存の提出・修正フローを含む182テストが成功した。</x:v>
       </x:c>
       <x:c r="I89" s="211" t="str">
-        <x:v>認証済みE2Eで3段階の一部不正解、修正再提出、全問合格、履歴、進捗を検証する。</x:v>
+        <x:v>QAテスト利用者でSTEP 1の進級テストと、STEP 2・3・4の固定問題消費後を開き、入力・下書き・提出・履歴復元を実画面で確認する。</x:v>
       </x:c>
       <x:c r="J89" s="211" t="str">
         <x:v>決定的単体テスト、RLS、E2E、生成異常系が成功し、AI上限について所有者の明示承認を得る</x:v>
       </x:c>
       <x:c r="K89" s="211" t="str">
-        <x:v>web/src/**/*.test.ts / supabase/tests/ / web/e2e/</x:v>
+        <x:v>web/src/lib/features/learning/problem-generator.ts / problem-generator.test.ts / web/src/lib/features/learning/task-flow.ts</x:v>
       </x:c>
       <x:c r="L89" s="213" t="n">
-        <x:v>46271</x:v>
+        <x:v>46277</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="140" customHeight="1">
@@ -5357,10 +5386,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H90" s="211" t="str">
-        <x:v>14段階のうちSTEP 1を5問の文法基礎、STEP 2を3問の一文構成、STEP 3を3問の短い論理構成として再設計し、STEP 4の自力で意見と理由を書く段階へ接続。</x:v>
+        <x:v>14段階の学習順序を維持し、STEP 1を5種の基礎小問、STEP 2を一文構成3操作、STEP 3を論理の流れ3操作として各10セット個別設計。STEP 4以降の10論点も設問・根拠・反対意見を統一した。</x:v>
       </x:c>
       <x:c r="I90" s="211" t="str">
-        <x:v>実利用結果をもとに各セットの負荷・語彙・合格基準を再評価する。</x:v>
+        <x:v>実利用結果をもとに、問題文だけで題意を理解できるか、語彙と負荷が段階に合うかを継続確認する。</x:v>
       </x:c>
       <x:c r="J90" s="211" t="str">
         <x:v>画面・設計書・問題生成で14段階が一致する</x:v>
@@ -5369,7 +5398,7 @@
         <x:v>docs/architecture.md / web/scripts/convert-curriculum.ts / web/src/lib/data/curriculum.json</x:v>
       </x:c>
       <x:c r="L90" s="213" t="n">
-        <x:v>46271</x:v>
+        <x:v>46275</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="140" customHeight="1">
@@ -5395,22 +5424,22 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H91" s="211" t="str">
-        <x:v>STEP 1の5問セットに加え、STEP 2・3の3問セットを画面・Claude採点・修正・履歴・問題識別へ実装。旧未提出課題だけ現行版へ更新し、提出済み履歴は変更しない。</x:v>
+        <x:v>STEP 1の不自然な「私は読書がを続けている」を、実際に起こり得る「図書館で通っている」から「図書館に通っている」へ直す助詞問題へ変更。固定問題版をadaptive-local-v14へ更新し、未提出の旧問題を現行内容へ更新できるようにした。</x:v>
       </x:c>
       <x:c r="I91" s="211" t="str">
-        <x:v>認証済みE2Eで選択式・記述式・下書き復元と3問セットの一連操作を確認する。</x:v>
+        <x:v>公開画面で新しい助詞問題の表示・選択・提出・解説を確認する。</x:v>
       </x:c>
       <x:c r="J91" s="211" t="str">
         <x:v>5問をまとめて提出でき、正誤・正解・理由が全問表示される</x:v>
       </x:c>
       <x:c r="K91" s="211" t="str">
-        <x:v>web/src/routes/tasks/[taskId]/+page.svelte / web/src/lib/features/learning/feedback.ts</x:v>
+        <x:v>web/src/lib/features/learning/curated-question-sets.ts / learning-design.ts / problem-generator.test.ts</x:v>
       </x:c>
       <x:c r="L91" s="213" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92" ht="150" customHeight="1">
+        <x:v>46277</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="155" customHeight="1">
       <x:c r="A92" s="211" t="str">
         <x:v>DB-011</x:v>
       </x:c>
@@ -5433,10 +5462,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H92" s="211" t="str">
-        <x:v>段階上限制約と進級RPCを14へ拡張済み。未提出の旧STEP 2・3だけを現行問題へ更新するmigrationに続き、別段階の未提出課題を保持したまま到達済み段階へ移動できるmigrationを適用。提出済み履歴・未提出課題はいずれも削除しない。</x:v>
+        <x:v>最高到達段階のフェーズ・合格数・受験数を保存する列と保護トリガーを追加。最高到達段階は減少不可とし、復習中の提出も先の段階の解放状態を変更しない。進級成立時は同一トランザクション内で次段階を解放する。</x:v>
       </x:c>
       <x:c r="I92" s="211" t="str">
-        <x:v>認証済みE2Eで未提出課題がある状態の段階変更と、元の段階へ戻った際の課題再開を確認する。</x:v>
+        <x:v>認証済みE2Eで進級直後・ページ移動後・復習後のDB値が一致することを確認する。</x:v>
       </x:c>
       <x:c r="J92" s="211" t="str">
         <x:v>段階14を保存でき、段階1の答え公開後に同じセットを再提出できない</x:v>
@@ -5445,10 +5474,10 @@
         <x:v>supabase/migrations/202609020001_fourteen_stage_curriculum.sql / 202609020002_stage_one_skill_targets.sql / 202609020003_expand_skill_allowlist.sql</x:v>
       </x:c>
       <x:c r="L92" s="213" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="150" customHeight="1">
+        <x:v>46272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="155" customHeight="1">
       <x:c r="A93" s="211" t="str">
         <x:v>QA-011</x:v>
       </x:c>
@@ -5471,10 +5500,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H93" s="211" t="str">
-        <x:v>STEP 1の5問とSTEP 2・3の3問セットについて、件数・カテゴリ・問題ハッシュ・全問正解・修正再提出・履歴・27セット重複回避を122単体テストで検証。未提出課題を保持した段階変更のDB契約テストを追加し、123テスト、型検査、製品ビルド、migration適用が成功。</x:v>
+        <x:v>全STEP 1〜13について進級テストの規定合格到達直後に次段階が解放されることを単体検証。復習前後の進級状態保存・復元とDB契約を追加し、127テスト、型検査、製品ビルド、migration適用が成功。</x:v>
       </x:c>
       <x:c r="I93" s="211" t="str">
-        <x:v>認証済み画面E2EでClaude実応答、DB保存、履歴、進捗、未提出課題を残した段階往復を確認する。</x:v>
+        <x:v>認証済み画面E2EでSTEP 4から5と、別の代表段階の進級・復習往復を確認する。</x:v>
       </x:c>
       <x:c r="J93" s="211" t="str">
         <x:v>ローカル・DBで段階数、採点、進級、履歴が一致する</x:v>
@@ -5483,10 +5512,10 @@
         <x:v>web/src/**/*.test.ts / supabase/tests/learner_data_rls.sql</x:v>
       </x:c>
       <x:c r="L93" s="213" t="n">
-        <x:v>46271</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94" ht="130" customHeight="1">
+        <x:v>46272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="145" customHeight="1">
       <x:c r="A94" s="211" t="str">
         <x:v>AI-009</x:v>
       </x:c>
@@ -5509,19 +5538,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H94" s="211" t="str">
-        <x:v>暫定上限をDBで強制し、呼出前予約と利用量記録を実装。Schema修正後のSonnet 4.6直接検査は入力924・出力331トークン。現行上限値は未承認のprovisional。</x:v>
+        <x:v>問題生成に加え、独立品質審査と不合格時1回だけの修正生成について暫定予算・日次回数・実使用量記録を追加。品質審査は入力14,000・出力2,200、1日6回、修正生成は入力18,000・出力3,500、1日3回の暫定安全値とし、ai_usage_eventsへ工程別に記録する。</x:v>
       </x:c>
       <x:c r="I94" s="211" t="str">
-        <x:v>利用者画面の実提出でトークン量を記録し、最終リリーステストで品質・費用を提示して上限変更を必ず確認する。</x:v>
+        <x:v>実生成で各工程の入力・出力トークン、応答時間、1問当たり費用、修正発生率、品質を測定する。最終リリーステストで問題生成・審査・修正・添削の暫定上限をサービス責任者へ必ず確認する。</x:v>
       </x:c>
       <x:c r="J94" s="211" t="str">
         <x:v>暫定値を本番へ流用せず、所有者確認済みの上限で品質・費用テストが成功しreview_statusがapprovedになる</x:v>
       </x:c>
       <x:c r="K94" s="211" t="str">
-        <x:v>web/src/lib/features/learning/ai-budget.ts / supabase/migrations/202608210001_initial_schema.sql</x:v>
+        <x:v>supabase/functions/problem-generation/index.ts / supabase/migrations/202609110003_generated_problem_quality_lifecycle.sql / docs/architecture.md</x:v>
       </x:c>
       <x:c r="L94" s="213" t="n">
-        <x:v>46271</x:v>
+        <x:v>46276</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="140" customHeight="1">
@@ -5585,19 +5614,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H96" s="211" t="str">
-        <x:v>STEP 2を情報関係・曖昧さ・情報選択、STEP 3を順序・不足説明・流れ修正の平易な3問セットへ更新。各問題は改行表示し、記述問題には複数行入力欄を使う。</x:v>
+        <x:v>STEP 2の情報選択10問を再調整。問題の条件は維持しながら、指示を原則1文・最大2文に短縮した。「中心となる」を繰り返す表現を削除し、見出しを意見・目的・方針・話題へ簡潔化。解説も選ぶ材料と除く材料だけを端的に示す表現へ統一した。</x:v>
       </x:c>
       <x:c r="I96" s="211" t="str">
-        <x:v>Claudeの実コメントが学習者に分かりやすい日本語か確認し、必要なら表現を調整する。</x:v>
+        <x:v>公開画面でSTEP 2の10セットを確認し、短い指示だけで使う材料と除く材料が迷わず分かるか評価する。</x:v>
       </x:c>
       <x:c r="J96" s="211" t="str">
         <x:v>課題文だけで入力形式を判断でき、ヒント・解答例・採点条件が矛盾しない</x:v>
       </x:c>
       <x:c r="K96" s="211" t="str">
-        <x:v>web/scripts/practice-bank.ts / web/src/lib/features/learning/learning-design.ts / feedback.ts</x:v>
+        <x:v>web/src/lib/features/learning/curated-question-sets.ts / problem-generator.test.ts / docs/architecture.md</x:v>
       </x:c>
       <x:c r="L96" s="213" t="n">
-        <x:v>46271</x:v>
+        <x:v>46277</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5630,7 +5659,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d6ad80f984b4e34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcca89c8d1d7248bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5969,38 +5998,38 @@
     </x:row>
     <x:row r="20" ht="92" customHeight="1">
       <x:c r="A20" s="230" t="n">
-        <x:v>46261</x:v>
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="B20" s="224" t="str">
-        <x:v>再提出・進級ループ・画面改善</x:v>
+        <x:v>AI問題生成</x:v>
       </x:c>
       <x:c r="C20" s="224" t="str">
-        <x:v>要修正答案の修正・再提出、問題切替時の表示リセット、通常訓練→進級テスト→再訓練→再受験、3種類の回数設定、ホーム・課題・アカウント画面の文言とアイコンを実装</x:v>
+        <x:v>問題生成の標準モデルをSonnet 5へ変更し、添削モデル設定と分離。段階設計に沿う生成プロンプト、素材の扱い・追加条件・複数解答例・技能別合格条件・隠れた採点条件なしを持つ構造化Schema、保存前の整合性検証、共通生成関数を追加した。</x:v>
       </x:c>
       <x:c r="D20" s="224" t="str">
-        <x:v>APP-003〜004・007〜008・012・014 / DB-008 / QA-008〜009</x:v>
+        <x:v>AI-004・006・008・009 / QA-009</x:v>
       </x:c>
       <x:c r="E20" s="224"/>
       <x:c r="F20" s="224" t="str">
-        <x:v>開発DBへmigration適用、2ユーザーRLS/RPC実測成功。pnpm verify成功（7ファイル・53テスト、型0警告、製品ビルド成功）</x:v>
+        <x:v>149テスト・型検査成功。問題生成Edge Function、予算予約、再生成、問題バンク登録、実API評価は次工程。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="78" customHeight="1">
       <x:c r="A21" s="230" t="n">
-        <x:v>46261</x:v>
+        <x:v>46275</x:v>
       </x:c>
       <x:c r="B21" s="224" t="str">
-        <x:v>活動グリッド表示修正</x:v>
+        <x:v>論点拡張・自由テーマ設定</x:v>
       </x:c>
       <x:c r="C21" s="224" t="str">
-        <x:v>DB上の提出3件と日時を確認。狭幅画面で1月位置が初期表示され、8月の活動マスが横スクロール外に隠れる問題を修正し、最新活動週を自動表示</x:v>
+        <x:v>STEP 4〜14を大学入試小論文向け78論点へ拡張。設定画面に初期値ランダムと、1〜3件・各20文字以内の自由設定を追加した。自由テーマはSTEP 4以降の次問から反映し、テーマ固有IDで固定論点や別テーマとの混在を防止。Claude問題生成へ同じテーマを渡し、DBにも制約付きで保存する。</x:v>
       </x:c>
       <x:c r="D21" s="224" t="str">
-        <x:v>APP-011 / QA-007</x:v>
+        <x:v>APP-004・013 / CUR-005〜007 / DB-005・010 / AI-008 / OPS-002 / QA-001・009〜010</x:v>
       </x:c>
       <x:c r="E21" s="224"/>
       <x:c r="F21" s="224" t="str">
-        <x:v>pnpm check成功、53テスト成功。提出データの削除・変更なし</x:v>
+        <x:v>18ファイル166テスト、型検査0エラー・0警告、製品ビルド成功。migration 202609100001をオンライン適用し、problem-generation-v3とCloudflare Version 2d3748d9-dce0-4e83-bb08-53c13e10907cを公開。認証済み自由テーマE2Eは次回確認。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="84" customHeight="1">
@@ -6901,6 +6930,438 @@
       <x:c r="E71" s="211"/>
       <x:c r="F71" s="211" t="str">
         <x:v>123テスト・型検査・製品ビルド成功。Supabase migration 202609060003_allow_stage_switch_with_open_problem.sqlを適用し、本番関数が未提出課題で段階変更を拒否しないことを確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="190" customHeight="1">
+      <x:c r="A72" s="213" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="B72" s="211" t="str">
+        <x:v>進級状態を復習・画面移動から保護</x:v>
+      </x:c>
+      <x:c r="C72" s="211" t="str">
+        <x:v>到達済み段階を選ぶと最高到達段階の進級テスト状態と合格数が失われる全段階共通の不具合を修正。最高到達段階の状態を別に保存し、復習後に復元する。最高到達段階は減少不可とし、進級成立と同じDB処理内で次段階を解放する。画面状態も完了・復習中・学習中・未完了へ整理した。</x:v>
+      </x:c>
+      <x:c r="D72" s="211" t="str">
+        <x:v>APP-007〜008 / DB-011 / OPS-002 / QA-001・011</x:v>
+      </x:c>
+      <x:c r="E72" s="211"/>
+      <x:c r="F72" s="211" t="str">
+        <x:v>127テスト・型検査・製品ビルド成功。Supabase migration 202609070001_preserve_frontier_progress.sqlを適用。Cloudflare Version bf7116ff-7f98-473f-ba24-5402c8e7f5f1、公開課題ページHTTP 200。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="160" customHeight="1">
+      <x:c r="A73" s="207" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="B73" s="207" t="str">
+        <x:v>Claude添削</x:v>
+      </x:c>
+      <x:c r="C73" s="207" t="str">
+        <x:v>要修正の結果画面でだけ「やさしい説明を見る」を追加。Claude Haikuが元の添削を小学校高学年〜中学生向けに言い換えるが、合否・進級・正式添削は変更しない。同一提出IDの結果は保存して再利用し、入力2,600・出力600トークン、1日5回の暫定上限をDBで強制する。</x:v>
+      </x:c>
+      <x:c r="D73" s="207" t="str">
+        <x:v>AI-003・006・007・009 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E73" s="207"/>
+      <x:c r="F73" s="207" t="str">
+        <x:v>129テスト、型検査、製品ビルド成功。Supabase migration 202609070002とsimplify-feedback Functionを適用。Cloudflare Version b6fd461d-2479-49d5-8b43-e8a4217ae202へ公開。実Claude品質・実測トークンは次の利用者テストで確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="120" customHeight="1">
+      <x:c r="A74" s="233" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="B74" s="207" t="str">
+        <x:v>毎回のやさしい解説設定</x:v>
+      </x:c>
+      <x:c r="C74" s="207" t="str">
+        <x:v>進捗・設定画面へ難易度スイッチを追加。ONでは通常のClaude添削1回の解説を小学校高学年〜中学生向けにし、合否・採点基準・進級は維持する。設定を本人のlearning_progressへ保存し、添削関数がサーバー側で読み取る。ON時は重複するオンデマンド説明ボタンを隠す。</x:v>
+      </x:c>
+      <x:c r="D74" s="207" t="str">
+        <x:v>APP-004 / DB-005 / AI-003・005〜006・009 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E74" s="207"/>
+      <x:c r="F74" s="207" t="str">
+        <x:v>133テスト、型検査、製品ビルド、Supabase Claude権限/RLSテスト成功。migration 202609070003とfeedback Functionを配備。Cloudflare Version 9ef36a4c-e2bd-4aec-87d5-93059f7ba3fd、公開/progress HTTP 200。実Claude品質・実測トークンは利用者テストで確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="120" customHeight="1">
+      <x:c r="A75" s="233" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="B75" s="207" t="str">
+        <x:v>進捗・設定画面の案内文調整</x:v>
+      </x:c>
+      <x:c r="C75" s="207" t="str">
+        <x:v>ページタイトルを「学習進捗・設定」へ変更。解説の難易度をONにした場合は、読みやすさを優先するため解説が長くなったり最適な表現から若干ズレる可能性があることを、合否や採点基準は変わらない旨とともに明記した。</x:v>
+      </x:c>
+      <x:c r="D75" s="207" t="str">
+        <x:v>APP-004 / AI-005 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E75" s="207"/>
+      <x:c r="F75" s="207" t="str">
+        <x:v>133テスト、型検査、製品ビルド成功。Cloudflare Version 04a67cd6-a884-477b-a840-dde540087086へ公開し、公開/progressのHTTP 200を確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="120" customHeight="1">
+      <x:c r="A76" s="233" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="B76" s="207" t="str">
+        <x:v>やさしい解説の修正画面引継ぎ</x:v>
+      </x:c>
+      <x:c r="C76" s="207" t="str">
+        <x:v>オンデマンドのやさしい解説を表示してから修正へ進む場合、その解説と「次にすること」を入力欄の上へ表示するよう変更。未取得なら通常解説を転記する。単問と問題セットの両方に対応し、再読み込み時はSupabaseの保存済み結果だけを取得してClaudeの追加利用を防ぐ。</x:v>
+      </x:c>
+      <x:c r="D76" s="207" t="str">
+        <x:v>APP-006・007 / AI-003 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E76" s="207"/>
+      <x:c r="F76" s="207" t="str">
+        <x:v>17ファイル134テスト、型検査0エラー・0警告、製品ビルド成功。Cloudflare Version bdac8222-6f6b-4ee5-94a6-6ab8150776f7へ公開し、公開/tasks HTTP 200を確認。実アカウントE2Eは次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="120" customHeight="1">
+      <x:c r="A77" s="233" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+      <x:c r="B77" s="207" t="str">
+        <x:v>複数問題の解説・解答レイアウト</x:v>
+      </x:c>
+      <x:c r="C77" s="207" t="str">
+        <x:v>STEP 1〜3の問題セットで、解説を画面上部に一括表示する構成を廃止。修正画面は各問題の「問題文→解説→入力欄」、結果画面は「問題文→あなたの解答→正誤→解説」を1カードにまとめた。やさしい解説を取得済みの場合も、対応する不正解問題のカードだけに表示する。</x:v>
+      </x:c>
+      <x:c r="D77" s="207" t="str">
+        <x:v>APP-007 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E77" s="207"/>
+      <x:c r="F77" s="207" t="str">
+        <x:v>17ファイル135テスト、型検査0エラー・0警告、製品ビルド成功。Cloudflare Version 0a495e9a-33e9-4248-8045-b45acbb8a9e5へ公開し、公開/tasks HTTP 200を確認。認証済み画面E2Eは次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="120" customHeight="1">
+      <x:c r="A78" s="233" t="n">
+        <x:v>46273</x:v>
+      </x:c>
+      <x:c r="B78" s="207" t="str">
+        <x:v>全段階のClaude添削整合性修正</x:v>
+      </x:c>
+      <x:c r="C78" s="207" t="str">
+        <x:v>STEP 1〜3で学習者解答と正解資料を明示分離し、Claudeが不正解としながら正解例に同じ答案を示す場合は正解へ補正して解説も整合させる。セット合否は各問から再計算。STEP 4〜14には合否・言語状態・技能評価・未回答説明の矛盾検査を追加。問題識別値へ採点資料を含め、問題版をv10へ更新した。</x:v>
+      </x:c>
+      <x:c r="D78" s="207" t="str">
+        <x:v>APP-007 / AI-003・005・006 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E78" s="207"/>
+      <x:c r="F78" s="207" t="str">
+        <x:v>17ファイル138テスト、型検査0エラー・0警告、製品ビルド成功。feedback Edge FunctionをSupabaseへ、Cloudflare Version cf7b66aa-530c-4e27-8e3d-25bb74a6cc64を検証環境へ公開。トップ・課題画面HTTP 200。認証済み全段階E2Eは次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="120" customHeight="1">
+      <x:c r="A79" s="233" t="n">
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="B79" s="207" t="str">
+        <x:v>やさしい解説を設定方式へ一本化</x:v>
+      </x:c>
+      <x:c r="C79" s="207" t="str">
+        <x:v>結果後の「やさしい説明を見る」と追加Claude呼出を廃止。設定OFFは通常解説、ONは小学校高学年〜中学生向け解説のどちらか一種類だけを通常添削で生成・表示・保存する。課題トップの取り組むボタン付近とOFF時の要修正結果に設定案内を追加。専用Edge Function、DB関数、キャッシュテーブル、予算設定を撤去した。</x:v>
+      </x:c>
+      <x:c r="D79" s="207" t="str">
+        <x:v>APP-006・007 / AI-003・005・006 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E79" s="207"/>
+      <x:c r="F79" s="207" t="str">
+        <x:v>17ファイル138テスト、型検査0エラー・0警告、製品ビルド、migration dry-run成功。migration適用とsimplify-feedback削除後、DB撤去対象不在・通常feedback ACTIVEを確認。Cloudflare Version a783c524-4627-4f87-8b7a-7d8a2d5f9868へ公開し、3画面HTTP 200。実アカウントE2Eは次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="120" customHeight="1">
+      <x:c r="A80" s="233" t="n">
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="B80" s="207" t="str">
+        <x:v>複数問題の入力見積りとエラー表示を修正</x:v>
+      </x:c>
+      <x:c r="C80" s="207" t="str">
+        <x:v>STEP 1〜3は各問題、正解候補、採点観点、出力Schema、やさしい表現指示を含むClaude要求全体をUTF-8バイト数から見積もる。全段階で呼出直前にも再検査する。添削暫定値を入力8,000・出力1,800・1日20回・日次入力160,000へ調整。やさしい解説は通常添削と同じ1回で生成し、専用回数なし。80文字までの安全なエラーコードと原因別メッセージへ対応した。</x:v>
+      </x:c>
+      <x:c r="D80" s="207" t="str">
+        <x:v>AI-003・007 / OPS-002 / QA-001</x:v>
+      </x:c>
+      <x:c r="E80" s="207"/>
+      <x:c r="F80" s="207" t="str">
+        <x:v>17ファイル141テスト、型検査0エラー・0警告、製品ビルド、migration dry-run・適用、Claude予約DBロールバックテスト、公開3画面HTTP 200に成功。feedback Version 10、Cloudflare Version d4f2eb9f-72b8-46b3-b315-15291da2e288。DBで暫定上限とやさしい解説専用予算なしを確認。実アカウントE2Eは次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="135" customHeight="1">
+      <x:c r="A81" s="233" t="n">
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="B81" s="207" t="str">
+        <x:v>カリキュラム・AI添削</x:v>
+      </x:c>
+      <x:c r="C81" s="207" t="str">
+        <x:v>問題文と採点条件の不整合を修正</x:v>
+      </x:c>
+      <x:c r="D81" s="207" t="str">
+        <x:v>AI-003 / CUR-006 / QA-001</x:v>
+      </x:c>
+      <x:c r="E81" s="207"/>
+      <x:c r="F81" s="207" t="str">
+        <x:v>STEP 1〜14の課題構造を確認。STEP 2の主語が特定できない問題と、STEP 3の元情報の扱いが曖昧な3問題を修正。正解例だけを暗黙の必須条件にしない採点規則と回帰テストを追加。143件の自動テスト、型検査、製品ビルドに成功。Supabase feedback Version 11、Cloudflare Version 4b671d6a-5825-46f4-83ec-a5424e7653aaへ公開し、課題トップHTTP 200を確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="n">
+        <x:v>46274</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>Claude問題生成を全14段階へ接続・公開</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>固定問題と承認済み問題バンクを優先し、在庫がない場合だけSonnet 5で生成する仕組みを実装。段階別Schemaと再検証、検証不合格時1回再生成、安定request_id、暫定予算予約、問題バンク登録・再利用、発行、利用量記録、失敗時のローカル問題退避を追加した。</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>AI-004・006〜009 / DB-010 / OPS-002 / QA-001・009〜010</x:v>
+      </x:c>
+      <x:c r="E82"/>
+      <x:c r="F82" t="str">
+        <x:v>18ファイル152テスト、型検査0エラー・0警告、製品ビルド成功。migration 202609090003をオンライン適用しproblem-generation Functionを配備。CORS 204・未認証401。Cloudflare Version ede05f22-7d34-4728-ba13-224ab6d3b830、公開4画面HTTP 200。実ユーザー生成品質・実測費用は要確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="190" customHeight="1">
+      <x:c r="A83" s="213" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="B83" s="211" t="str">
+        <x:v>固定問題10セットと後半課題の品質監査・修正</x:v>
+      </x:c>
+      <x:c r="C83" s="211" t="str">
+        <x:v>STEP 1の5問×10セット、STEP 2・3の3問×10セットを個別設計し、全110小問の日本語・指示・正解・解説を確認。STEP 4〜14は10の共通論点を統一し、元情報の扱い、結論、反対意見への応答などの提出条件を明記した。固定例を問題の正解と誤認しない表示も追加した。</x:v>
+      </x:c>
+      <x:c r="D83" s="211" t="str">
+        <x:v>CUR-005〜009 / APP-013 / QA-009〜010</x:v>
+      </x:c>
+      <x:c r="E83" s="211" t="str"/>
+      <x:c r="F83" s="211" t="str">
+        <x:v>全157テスト、Svelte型検査0エラー・0警告、Cloudflare製品ビルド成功。feedback・problem-generationをSupabaseへ、Cloudflare Version 22dd4bdf-0267-487a-9513-aa175ec7abb3を検証環境へ公開。公開3画面HTTP 200、問題生成関数CORS 204・未認証401。実アカウントでの代表問題とClaude生成品質は次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>論点拡張・自由テーマ設定</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>STEP 4〜14を大学入試小論文向け78論点へ拡張。設定画面に初期値ランダムと、1〜3件・各20文字以内の自由設定を追加した。自由テーマはSTEP 4以降の次問から反映し、テーマ固有IDで固定論点や別テーマとの混在を防止。Claude問題生成へ同じテーマを渡し、DBにも制約付きで保存する。</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>APP-004・013 / CUR-005〜007 / DB-005・010 / AI-008 / OPS-002 / QA-001・009〜010</x:v>
+      </x:c>
+      <x:c r="E84"/>
+      <x:c r="F84" t="str">
+        <x:v>18ファイル166テスト、型検査0エラー・0警告、製品ビルド成功。migration 202609100001をオンライン適用し、problem-generation-v3とCloudflare Version 323154c0-dea6-482f-9bd5-d7b2c282cd04を公開。認証済み自由テーマE2Eは次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>提出中断後の結果復旧</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>提出返答前にスクリーンセーバーや認証更新で画面処理が止まっても、同一タブに保持した提出IDで完了を自動確認する。サーバー側で保存済みなら、問題・解答・添削・提出前進捗から結果画面を再構成する。古い問題URLで別の未提出問題が現在問題の場合は自動移動する。</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>APP-007 / QA-001 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E85"/>
+      <x:c r="F85" t="str">
+        <x:v>18ファイル169テスト、型検査0エラー・0警告、製品ビルド成功。Cloudflare Version 23d684e6-2040-4cae-8d02-7415b8890400へ公開し、課題画面とService WorkerのHTTP 200を確認。実アカウントでのスリープ復旧再現テストは次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>復習ボタンの直接遷移</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>課題トップの「復習する」または「学習に戻る」を押した際、段階変更の保存後に対象段階の未提出問題または次の問題を選び、その問題画面へ直接移動するよう変更した。最上部へ戻って「取り組む」を押す二重操作をなくした。</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>APP-004 / QA-001 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E86"/>
+      <x:c r="F86" t="str">
+        <x:v>18ファイル170テスト、型検査0エラー・0警告、製品ビルド成功。Cloudflare Version 1e1637d1-13fc-4e18-840b-4c6808787f74へ公開。実アカウントでの復習直接遷移は次回確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="n">
+        <x:v>46275</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>Claude添削の判定整合性を修正</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>ClaudeがlanguageStatusをclean、decisionをreviseと返した際にinconsistent_decisionとして保存を止めていた過剰検証を修正。日本語表現の状態と段階目標の達成判定を分離し、DBと同じ規則へ統一した。Claude指示と回帰テストを追加し、応答後の検証失敗でも実使用量を記録するよう修正した。</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>AI-003・006 / QA-001</x:v>
+      </x:c>
+      <x:c r="E87"/>
+      <x:c r="F87" t="str">
+        <x:v>18ファイル171テスト、型検査0エラー・0警告、製品ビルド成功。feedback Edge FunctionをSupabaseへ配備。実アカウントで同じ答案の再提出確認が必要。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>固定問題消費後のClaude生成QAハーネス</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>通常の画面・URL・出題経路を変えず、テスト利用者だけの固定問題10セット消費済み状態を作るローカル専用ツールを追加。生成問題はqa状態で隔離し、通常利用者には出題されない。リセットは当該利用者の下書き・提出・添削・履歴・AI利用記録とqa問題だけを削除する。</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>QA-010 / AI-008〜009 / DB-010</x:v>
+      </x:c>
+      <x:c r="E88"/>
+      <x:c r="F88" t="str">
+        <x:v>QAハーネスのDB migrationをSupabaseへ適用。172テスト、型検査0エラー・0警告、製品ビルド成功。テスト用メールの登録・確認後にseed、Claude生成、添削、履歴復元、resetを実アカウントで確認する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>QAハーネスのSolレビュー修正とDB統合テスト</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>QA問題を履歴より先に削除する外部キー不整合、進捗保護トリガーにより最高到達段階が戻らない問題、QA本文ハッシュと通常問題の衝突、QA接尾辞を自由テーマとして解釈する問題を修正。使い捨て利用者で投入・隔離・生成確定・完全リセットを検証するSQLテストを追加した。</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>QA-010 / AI-008〜009 / DB-010</x:v>
+      </x:c>
+      <x:c r="E89"/>
+      <x:c r="F89" t="str">
+        <x:v>migration 202609110002をSupabaseへ適用。QA統合テストと既存RLS回帰テストがロールバックまで成功。173テスト、型検査0エラー・0警告、製品ビルド成功。Cloudflare Version 1e5100c2-a14e-4aff-a45d-adc9b3c333adへ公開し、トップ・課題画面HTTP 200。実Claudeテストはメール登録後に実施する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="55" t="n">
+        <x:v>46276</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>生成問題の事前品質審査・試行運用・5回終了</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>Claude生成直後に別呼出で7項目を第三者審査し、不合格時は1回だけ修正して再審査する。合格前はtrialとして共有せず、5回目の要修正で問題を不採用にして模範解答を示し、進捗へ不利益を与えず次問へ進める。5回未満で正しく解答できた共通テーマ問題だけ共有問題バンクへ昇格し、自由テーマは共有しない。</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>AI-008〜009 / DB-010 / QA-001・010 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E90"/>
+      <x:c r="F90" t="str">
+        <x:v>migration 202609110003をオンライン適用し、problem-generation Edge FunctionとCloudflare Version 5076f2b8-5ea4-4fc8-b68a-17b0403a4911を公開。18ファイル178テスト、型検査、製品ビルド、品質ライフサイクル・既存RLS・Claude・QAのDB統合テストが成功。トップ・課題一覧HTTP 200。実Claude生成と5回終了の認証済みE2Eは要確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="55" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>STEP 1助詞問題と進級テスト入力ロックを修正</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>不自然な助詞の連続を題材にした問題を、実際に起こり得る助詞選択の誤りへ変更した。固定問題消費後のClaude試用・QA問題ではURL識別子が復元時に失われ、DBの発行済み問題IDと一致せず入力がロックされていたため、解析後も元のIDを保持するよう共通処理を修正した。</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>APP-016 / AI-008 / QA-001・010 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E91"/>
+      <x:c r="F91" t="str">
+        <x:v>STEP 1〜14、選択式・記述式、自由テーマ、trial・QA識別子を回帰検査。18ファイル182テスト、型検査0エラー・0警告、製品ビルド成功。Cloudflare Version 4e282319-fc91-42b7-9520-8f2c7a0c20faへ公開し、トップ・課題一覧HTTP 200。認証済み実画面でのSTEP 1進級テスト操作は要確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="55" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>STEP 2情報選択問題の指示を全面改訂</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>「目的・方法・補足」の関係と補足の扱いを学習者へ推測させていたため、固定10問を中心内容と番号付き材料の形式へ統一した。必ず残す内容、使う材料、使わない材料、言い換えの可否を明記した。Claude生成問題にも同じ構造検査と独立品質審査を適用した。</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>CUR-011 / AI-008 / QA-001 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E92"/>
+      <x:c r="F92" t="str">
+        <x:v>18ファイル185テスト、型検査0エラー・0警告、製品ビルド成功。Supabase problem-generationとCloudflare Version 6edcaaf1-af70-4343-bd35-1c492cfb679dへ公開。トップ・課題一覧HTTP 200。公開画面でのSTEP 2全10セットと実Claude生成品質は要確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="55" t="n">
+        <x:v>46277</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>STEP 2情報選択問題の説明を簡潔化</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>固定10問の指示・見出し・解説から説明の重複を削り、使う中心内容と材料、言い換え可を短い自然文で伝える形式へ統一した。Claude生成・入力検査・独立品質審査も同じ簡潔な形式に更新し、短くても材料の採否が曖昧な問題は拒否する。</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>CUR-011 / AI-008 / QA-001 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E93"/>
+      <x:c r="F93" t="str">
+        <x:v>18ファイル185テスト、型検査0エラー・0警告、製品ビルド成功。Supabase problem-generationとCloudflare Version eae4202e-ef18-4606-9c6f-ed577b9d9cffへ公開。トップ・課題一覧HTTP 200。公開画面と実Claude生成品質は要確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="55" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>進級テスト開始直後の入力ロックを修正</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>提出後の「次の問題へ」が、次問をDBで発行する前に画面だけ切り替えていたため、進級テスト開始直後は発行済み判定を満たさず入力がロックされていた。次問発行、状態再取得、発行済み確認、画面遷移の順に変更し、通常訓練・進級テスト・不合格後の次問へ共通適用した。</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>APP-012 / QA-001・008 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E94"/>
+      <x:c r="F94" t="str">
+        <x:v>関連4ファイル66テスト、全18ファイル186テスト、型検査0エラー・0警告、製品ビルド成功。Cloudflare Version d2f586f2-2e67-4e7e-abfb-9cf79bd2b46bへ公開し、トップ・課題一覧HTTP 200。認証済み実画面での進級テスト連続操作は要確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="55" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>提出結果の自動遷移競合を修正</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>STEP 2の要修正後合格で、進捗更新による自動遷移が結果画面より先に動き、解説を飛ばしてSTEP 3へ進む競合を修正した。保存済み結果の表示待ちを明示し、修正または次問を選ぶまで全段階で結果を復元する。添削コメント1〜5件を画面・DBの両方で必須にした。</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>APP-007・012 / DB-004 / QA-008 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E95"/>
+      <x:c r="F95" t="str">
+        <x:v>関連6ファイル73テスト、全18ファイル190テスト、型検査0エラー・0警告、製品ビルド成功。migration 202609150001をSupabaseへ適用。Cloudflare Version 21a2dec9-ff4e-42a6-b376-a1e8f1e6d6bcへ公開し、トップ・課題一覧HTTP 200。認証済み実画面でのSTEP 2再提出合格と代表経路は要確認。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6909,7 +7370,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R041fd1e859484e74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4c2d05d4c5740e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enable cumulative retries and revision-aware Claude feedback
</commit_message>
<xml_diff>
--- a/開発進捗管理.xlsx
+++ b/開発進捗管理.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="進捗サマリー" sheetId="1" r:id="Rc3ec61def1704ab9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="実装タスク" sheetId="2" r:id="Rdc585897afa5429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新履歴" sheetId="5" r:id="Rd1ff3e0bdd9c4670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="進捗サマリー" sheetId="1" r:id="Ra17bbac152b5474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="実装タスク" sheetId="2" r:id="Ra966ddc64eb54353"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新履歴" sheetId="5" r:id="Ra850c47d887247c7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1912,7 +1912,7 @@
     </x:row>
     <x:row r="22" ht="100" customHeight="1">
       <x:c r="A22" s="234" t="str">
-        <x:v>現在地: STEP 2で要修正後に合格すると、解説を表示せずSTEP 3へ進む不具合を修正した。原因は、提出保存で次段階が解放された直後に認証・DB状態の再読込が割り込み、未確認の提出結果より現在問題への自動遷移が優先される競合だった。全段階共通で、結果表示待ちを学習者が「解答を修正する」または「次の問題へ」を押すまで保持する。解説は1〜5件を必須とし、画面とDBの両方で0件を拒否する。全18ファイル190テスト、型検査、製品ビルドが成功。Supabase migration適用済み。Cloudflare Version 21a2dec9-ff4e-42a6-b376-a1e8f1e6d6bcへ公開し、トップ・課題一覧HTTP 200を確認。次は公開版でSTEP 2の要修正→再提出合格、一発合格、進級テスト合否の全経路で、解説確認後にのみ次へ進むことを確認する。最終テストでは問題生成・審査・修正・添削の暫定AI上限を所有者へ必ず確認する。</x:v>
+        <x:v>現在地: 複数問の進級テストを、一度に全問正解する方式から累積正解方式へ変更した。STEP 1〜3は正解済み小問を保持し、誤答だけを再提出できる。長文問題は前回答案を引き継ぎ、Claudeが直前の最優先修正点を先に確認するため、毎回ゼロから書き直さずに改善できる。ブラウザの申告ではなくDBの保存結果から正解済み小問と修正条件を取得する。18ファイル194テスト、型検査、製品ビルド、実Supabase RLSテストに成功。migration 202610200001とfeedback FunctionをSupabaseへ反映し、Cloudflare Version e56927af-7406-4a64-9915-3d42eb83ae01へ公開、トップ・課題一覧HTTP 200を確認した。次は公開版で複数問の累積合格、長文の修正後合格、再読込復元、生成trialの5回目終了を実Claudeで確認する。最終テストでは問題生成・審査・修正・添削の暫定AI上限を所有者へ必ず確認する。</x:v>
       </x:c>
       <x:c r="B22" s="234" t="str"/>
       <x:c r="C22" s="234" t="str"/>
@@ -1940,7 +1940,7 @@
     </x:row>
     <x:row r="24" ht="28" customHeight="1">
       <x:c r="A24" s="236" t="str">
-        <x:v>最終更新日: 2026-09-15　｜　進捗の正本: このファイル</x:v>
+        <x:v>最終更新日: 2026-10-20　｜　進捗の正本: このファイル</x:v>
       </x:c>
       <x:c r="B24" s="236" t="str"/>
       <x:c r="C24" s="236" t="str"/>
@@ -2572,10 +2572,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H17" s="84" t="str">
-        <x:v>要修正の再表示では、正式添削結果に保存された通常版またはやさしい版の一種類だけを入力欄の直前へ復元する。追加生成された別解説の読込と保存は廃止した。正解済み解答と下書きの復元は維持。</x:v>
+        <x:v>要修正後は、正解済みの小問・下書き・直前の解説に加え、長文問題の直前答案を復元する。複数問では正解済みを編集不可として保持し、誤答だけを直せる。長文では前回答案を初期値にし、同じ問題の最優先修正点を見ながら書き直せる。</x:v>
       </x:c>
       <x:c r="I17" s="84" t="str">
-        <x:v>実アカウントで設定OFF/ONそれぞれの要修正→画面再読込→再提出を行い、同じ一種類の解説と下書き・正解済み解答が保持されることを確認する。</x:v>
+        <x:v>公開版でSTEP 1〜3の一部だけを誤答して再読込し、正解済みが保持・固定され、誤答だけ再提出できることを確認する。STEP 13・14等の長文でも前回答案と直前の修正指示が復元されることを確認する。</x:v>
       </x:c>
       <x:c r="J17" s="77" t="str">
         <x:v>再読込後も下書きが復元される</x:v>
@@ -2584,7 +2584,7 @@
         <x:v>web/src/lib/features/learning/learning-service.ts / web/src/lib/features/learning/save-queue.ts / web/src/routes/tasks/</x:v>
       </x:c>
       <x:c r="L17" s="232" t="n">
-        <x:v>46274</x:v>
+        <x:v>46315</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="155" customHeight="1">
@@ -2610,10 +2610,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H18" s="84" t="str">
-        <x:v>正式提出・添削・書き直しに加え、提出成功後の結果表示待ち状態を同一タブへ保持する。要修正後の合格、一発合格、進級テストの合否は、認証・DB状態の再読込が起きても結果と解説を復元し、学習者が「解答を修正する」または「次の問題へ」を選ぶまで自動遷移しない。</x:v>
+        <x:v>通常トレーニングと進級テストの複数問を累積正解方式へ統一した。要修正では同じ問題を開いたまま、正解済みの小問を保持して誤答だけを再提出する。長文は直前答案を引き継ぎ、Claudeが前回の最優先修正点を先に確認する。修正できた答案へ新しい軽微な条件を追加して合格を先延ばししない指示も加えた。</x:v>
       </x:c>
       <x:c r="I18" s="84" t="str">
-        <x:v>認証済み公開画面でSTEP 2の要修正→修正→合格を行い、3問すべての解説を確認してから「次の問題へ」でSTEP 3へ進むことを確認する。あわせて一発合格と進級テストの合否でも同じ結果表示を確認する。</x:v>
+        <x:v>認証済み公開画面でSTEP 1〜3の進級テストを一部正解で提出し、誤答だけを複数回直して合格できることを確認する。長文は要修正→前回答案の修正→合格を確認し、再読込後も同じ状態が復元されることを確認する。</x:v>
       </x:c>
       <x:c r="J18" s="77" t="str">
         <x:v>提出状態と結果が永続化される</x:v>
@@ -2622,7 +2622,7 @@
         <x:v>web/src/routes/tasks/[taskId]/+page.svelte / web/src/lib/features/learning/submission-workflow.ts / progression.ts</x:v>
       </x:c>
       <x:c r="L18" s="232" t="n">
-        <x:v>46280</x:v>
+        <x:v>46315</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="155" customHeight="1">
@@ -3301,10 +3301,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H36" s="84" t="str">
-        <x:v>migration 202609050002を適用。STEP 1の不正解セットを閉じる特例を廃止。冪等性と進級テストの一回解答を維持。</x:v>
+        <x:v>migration 202610200001を適用。進級テストも要修正時は同じ発行問題を開いたままにし、修正提出を受け付ける。前回の要修正答案・添削結果をservice_role専用RPCで取得し、ブラウザ申告を信用せずサーバー側で正解済み小問と修正条件を確定する。生成問題の5回目終了規則は維持した。</x:v>
       </x:c>
       <x:c r="I36" s="84" t="str">
-        <x:v>既存の完了済み不合格セットは自動で再開しない。新規提出から仕様を適用する。</x:v>
+        <x:v>今後のDB変更も新しいmigrationとして追加する。認証済み公開画面で、進級テストの修正中に再読込しても同じ問題・正解済み小問・直前答案が復元されることを確認する。</x:v>
       </x:c>
       <x:c r="J36" s="77" t="str">
         <x:v>空の開発DBへ適用成功</x:v>
@@ -3313,7 +3313,7 @@
         <x:v>supabase/migrations/202608210001_initial_schema.sql / docs/supabase-local-setup.md</x:v>
       </x:c>
       <x:c r="L36" s="232" t="n">
-        <x:v>46270</x:v>
+        <x:v>46315</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="110" customHeight="1">
@@ -3532,10 +3532,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H42" s="84" t="str">
-        <x:v>feedback Edge Functionを更新し、languageStatus（日本語表現上の状態）とdecision（当該STEPの達成判定）を分離した。cleanかつreviseを正当な組み合わせとして許可し、revision_requiredかつpassは引き続き拒否する。Claudeへの指示、回帰テスト、検証失敗時の実使用量記録も追加し、Supabaseへ配備済み。</x:v>
+        <x:v>feedback Edge Functionをプロンプトv4へ更新。前回の要修正答案・添削をDBから取得し、複数問では正解済み小問を再採点せず固定する。長文では直前答案との差分と前回の最優先修正点を先に評価し、修正済みなら別の軽微な要求で不合格を続けない。Supabaseへ配備済み。</x:v>
       </x:c>
       <x:c r="I42" s="84" t="str">
-        <x:v>オンライン環境で同じ答案を再提出し、cleanかつreviseの判定が要修正結果として保存・表示されることを確認する。その後、STEP 2・3の自然な別解も確認する。</x:v>
+        <x:v>実Claudeで、複数問の一部正解保持と長文の要修正→修正後合格を確認する。同じ答案で判定が大きく揺れないこと、ブラウザから正解済みIDを偽装できないこと、生成問題の5回目終了が維持されることも確認する。</x:v>
       </x:c>
       <x:c r="J42" s="77" t="str">
         <x:v>正常・異常ケースがテストを通る</x:v>
@@ -3544,7 +3544,7 @@
         <x:v>supabase/functions/feedback/</x:v>
       </x:c>
       <x:c r="L42" s="232" t="n">
-        <x:v>46275</x:v>
+        <x:v>46315</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="145" customHeight="1">
@@ -4229,10 +4229,10 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H60" s="84" t="str">
-        <x:v>公式Cloudflareアダプター、Wrangler、Worker設定をweb内へ固定。製品build、dry-run、ローカルWorkersの主要画面で確認済み</x:v>
+        <x:v>公式Cloudflareアダプター、Wrangler、Worker設定をweb内へ固定。製品build、dry-run、ローカルWorkersの主要画面で確認済み Pagesは使用せず、Workers Static Assetsが画面と静的ファイルの配信を担う構成へ設計書を統一した。</x:v>
       </x:c>
       <x:c r="I60" s="84" t="str">
-        <x:v>Cloudflareの更新時に互換性とビルドを回帰確認する</x:v>
+        <x:v>Workers＋Workers Static Assets構成を維持する。一般公開前にTurnstileをOPS-004として実装し、最終デプロイと公開設定を確認する。</x:v>
       </x:c>
       <x:c r="J60" s="77" t="str">
         <x:v>Cloudflare向けbuildとローカルWorkers起動が成功する</x:v>
@@ -4241,7 +4241,7 @@
         <x:v>web/vite.config.ts / web/wrangler.jsonc / web/package.json</x:v>
       </x:c>
       <x:c r="L60" s="88" t="n">
-        <x:v>46268</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="145" customHeight="1">
@@ -5005,10 +5005,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H80" s="211" t="str">
-        <x:v>提出結果を未確認のまま自動遷移しない共通状態を追加。古い提出IDは30分で失効する一方、保存済み結果の表示待ちは学習者の操作まで保持する。空の解説を拒否し、最大5問の解説を受け入れる単体・画面・SQL契約テストを追加した。全18ファイル190テスト、型検査、製品ビルドが成功。</x:v>
+        <x:v>複数問の累積正解、進級テストの同一問題再提出、長文の直前答案・修正条件引継ぎ、サーバー側の正解済み判定を回帰テストへ追加した。18ファイル194テスト、型検査、製品ビルド、実Supabase RLSテストが成功。migration適用、feedback Function配備、Cloudflare Version e56927af-7406-4a64-9915-3d42eb83ae01への公開、トップ・課題一覧HTTP 200を確認した。</x:v>
       </x:c>
       <x:c r="I80" s="211" t="str">
-        <x:v>公開版でSTEP 2の要修正→再提出合格、STEP 1の5問合格、STEP 4以降の単問合格、進級テスト不合格・合格を操作し、すべて解説表示後にのみ遷移することを確認する。</x:v>
+        <x:v>公開版で①STEP 1〜3進級テストの一部誤答→誤答だけ再提出→累積合格、②長文の要修正→前回答案の一部修正→合格、③修正途中の再読込復元、④生成trialの5回目終了を実Claudeで確認する。</x:v>
       </x:c>
       <x:c r="J80" s="211" t="str">
         <x:v>ローカル・実DB・E2Eの主要境界ケースが成功する</x:v>
@@ -5017,7 +5017,7 @@
         <x:v>web/src/lib/features/learning/submission-workflow.ts / learning-service.ts / ui-copy.test.ts / sql-contract.test.ts</x:v>
       </x:c>
       <x:c r="L80" s="213" t="n">
-        <x:v>46280</x:v>
+        <x:v>46315</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="140" customHeight="1">
@@ -5310,19 +5310,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H88" s="211" t="str">
-        <x:v>Claudeのinformation_selection生成指示と構造検査を簡潔な自然文へ対応。問題文は意見・目的・方針・話題と番号付き材料を示し、2文以内で組み合わせ方と言い換え可を伝える。入力契約は短い有効表現を許可しつつ、使う材料と除く材料が不明な問題は引き続き拒否する。生成プロンプト版はproblem-generation-v5。</x:v>
+        <x:v>STEP 3固定問題から「〜という内容も残します」という重複説明を削除。Claude生成は、同じ扱いの素材を一度で指示し、個別素材の言い直しや修正経緯の名残を混ぜないよう変更した。構造検査で冗長な再説明を拒否し、独立品質審査でもblockingとして扱う。生成プロンプトはv6、品質審査はv3。</x:v>
       </x:c>
       <x:c r="I88" s="211" t="str">
-        <x:v>認証済みテスト利用者でSTEP 2の固定10セット後にClaude生成を実行し、簡潔さと採点条件の一致を確認する。</x:v>
+        <x:v>認証済みQA利用者でSTEP 3の固定問題消費後にClaude生成を実行し、問題文が簡潔で、素材・解答例・採点条件が一致することを確認する。生成問題、品質審査、AI使用履歴も確認する。</x:v>
       </x:c>
       <x:c r="J88" s="211" t="str">
         <x:v>不正・重複・条件逸脱問題を発行せず、生成コストと版を記録できる</x:v>
       </x:c>
       <x:c r="K88" s="211" t="str">
-        <x:v>supabase/functions/_shared/problem-generation-prompt.ts / problem-generation-contract.ts / problem-quality-prompt.ts</x:v>
-      </x:c>
-      <x:c r="L88" s="213" t="n">
-        <x:v>46277</x:v>
+        <x:v>web/src/lib/features/learning/curated-question-sets.ts / supabase/functions/_shared/problem-generation-prompt.ts / problem-generation-contract.ts / problem-quality-prompt.ts</x:v>
+      </x:c>
+      <x:c r="L88" s="213" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="145" customHeight="1">
@@ -5348,19 +5348,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H89" s="211" t="str">
-        <x:v>固定問題消費後のtrial問題IDから試用識別子が失われ、DBの発行済み問題と一致しないため入力がロックされる原因を特定・修正。STEP 1〜14、選択式・記述式、自由テーマ、QA識別子を同じ復元処理で検査し、既存の提出・修正フローを含む182テストが成功した。</x:v>
+        <x:v>固定問題消費QAを現行カリキュラム件数へ自動追随させ、STEP 1〜3は各10セット、STEP 4〜14は各78問を消費済みにする。対象STEPの承認済み共有問題も当該QA利用者の履歴上だけ消費済みにし、次問をClaude生成へ到達させる。QA専用ID、一般利用者との隔離、完全リセットを維持。</x:v>
       </x:c>
       <x:c r="I89" s="211" t="str">
-        <x:v>QAテスト利用者でSTEP 1の進級テストと、STEP 2・3・4の固定問題消費後を開き、入力・下書き・提出・履歴復元を実画面で確認する。</x:v>
+        <x:v>テスト用アカウントでseedを実行し、表示された固定問題数・共有問題数を確認する。通常アプリで次問を開き、problem_bank.status=qaとAI使用履歴、品質審査、添削、履歴復元、resetを実Claudeで確認する。</x:v>
       </x:c>
       <x:c r="J89" s="211" t="str">
         <x:v>決定的単体テスト、RLS、E2E、生成異常系が成功し、AI上限について所有者の明示承認を得る</x:v>
       </x:c>
       <x:c r="K89" s="211" t="str">
-        <x:v>web/src/lib/features/learning/problem-generator.ts / problem-generator.test.ts / web/src/lib/features/learning/task-flow.ts</x:v>
+        <x:v>tools/qa/qa-fixtures.mjs / tools/qa/seed-exhausted-stage.mjs / supabase/migrations/202610080001_dynamic_qa_exhaustion.sql / supabase/tests/qa_test_harness.sql</x:v>
       </x:c>
       <x:c r="L89" s="213" t="n">
-        <x:v>46277</x:v>
+        <x:v>46303</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="140" customHeight="1">
@@ -5659,7 +5659,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcca89c8d1d7248bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89d73951c7204fc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7364,13 +7364,67 @@
         <x:v>関連6ファイル73テスト、全18ファイル190テスト、型検査0エラー・0警告、製品ビルド成功。migration 202609150001をSupabaseへ適用。Cloudflare Version 21a2dec9-ff4e-42a6-b376-a1e8f1e6d6bcへ公開し、トップ・課題一覧HTTP 200。認証済み実画面でのSTEP 2再提出合格と代表経路は要確認。</x:v>
       </x:c>
     </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="55" t="n">
+        <x:v>46303</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>QA固定問題消費を現行カリキュラムへ追随</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>固定10件の前提を廃止し、各STEPの固定問題数を生成済みカリキュラムから取得するよう変更。STEP 4〜14の各78問と、対象STEPの承認済み共有問題をQA利用者の履歴上だけ消費済みにする。共有問題本体は変更せず、次問がClaude生成へ進む状態を作る。Cloudflare構成もPages不使用、Workers Static Assets利用へ文書を統一した。</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>QA-010 / AI-008〜009 / DB-010 / OPS-001〜004</x:v>
+      </x:c>
+      <x:c r="E96"/>
+      <x:c r="F96" t="str">
+        <x:v>migration 202610080001をSupabaseへ適用。QA統合テスト成功。18ファイル190テスト、QA fixture 2テスト、型検査0エラー・0警告、Cloudflare製品ビルド成功。実Claude生成、品質審査、添削、履歴復元、resetはテスト用アカウントで次に確認する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="55" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>STEP 3問題文の冗長表現を除去</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>固定問題の重複説明を削除した。Claude問題生成へ、同条件を一度で伝え、個別素材の言い直しや修正経緯を問題文へ混ぜない規則を追加した。構造検査で該当表現を拒否し、独立品質審査と修復指示でも簡潔な問題文へ統一する。</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>AI-008 / CUR-009 / QA-010 / OPS-002</x:v>
+      </x:c>
+      <x:c r="E97"/>
+      <x:c r="F97" t="str">
+        <x:v>Supabase problem-generation Functionへ反映済み。18ファイル191テスト、QA fixture 2テスト、型検査0エラー・0警告、Cloudflare製品ビルド成功。Cloudflare WorkersへのアップロードはWrangler OAuth再承認待ち。実Claude生成はQA利用者で要確認。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="112" customHeight="1">
+      <x:c r="A98" s="55" t="n">
+        <x:v>46315</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>進級テストの累積正解・長文の継続修正</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>通常トレーニングと進級テストの複数問で、正解済みを保持し誤答だけを再提出する方式へ統一した。長文は直前答案を引き継ぎ、前回の最優先修正点を先に評価する。前回結果はservice_role専用RPCから取得し、ブラウザによる正解済み判定の偽装を防ぐ。</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>APP-006・007 / DB-003 / AI-003 / QA-008</x:v>
+      </x:c>
+      <x:c r="E98"/>
+      <x:c r="F98" t="str">
+        <x:v>migration 202610200001を適用。feedback FunctionとCloudflare Version e56927af-7406-4a64-9915-3d42eb83ae01へ公開。18ファイル194テスト、型検査0エラー・0警告、製品ビルド、実Supabase RLSテスト、HTTP 200に成功。実Claudeによる公開画面確認は次の作業。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4c2d05d4c5740e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83d5968c3c2d495c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>